<commit_message>
Add daily test page + learning log: 2026-06-09
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,123 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>deleterious</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you hear about that old pesticide they stopped using? Turns out it had really deleterious effects on people's health—especially their lungs. So even though it worked great for keeping bugs away, the damage it caused was way worse. That's why companies need to think carefully before launching new products.</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>deleterious — 해로운, 유해한; launch — 출시하다, 출범하다</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R3" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S3" s="9" t="inlineStr"/>
+      <c r="T3" s="9" t="inlineStr"/>
+      <c r="U3" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V3" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W3" s="9" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="X3" s="9" t="inlineStr">
+        <is>
+          <t>마감 기한</t>
+        </is>
+      </c>
+      <c r="Y3" s="9" t="inlineStr">
+        <is>
+          <t>남북전쟁 포로수용소에서 그 선을 넘으면 사살한다는 경계선에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-10
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -885,6 +885,123 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: A Tale of Two Cities</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story, A Tale of Two Cities, and learn how English speakers use the word 'time' in different ways. You'll discover 15 useful expressions with 'time' that you can use in your daily conversations and business meetings. By the end of this lesson, you'll have a much better understanding of how native speakers talk about time.</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>explore — 탐험하다, 알아보다; expression — 표현, 표현법</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S4" s="9" t="inlineStr"/>
+      <c r="T4" s="9" t="inlineStr"/>
+      <c r="U4" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V4" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W4" s="9" t="inlineStr">
+        <is>
+          <t>bankrupt</t>
+        </is>
+      </c>
+      <c r="X4" s="9" t="inlineStr">
+        <is>
+          <t>파산한</t>
+        </is>
+      </c>
+      <c r="Y4" s="9" t="inlineStr">
+        <is>
+          <t>중세 환전상이 파산하면 거래 탁자(banca)를 부수는 관습에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-11
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1002,6 +1002,123 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>saturnine</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>My coworker has been really saturnine lately—always complaining and looking grumpy at meetings. I suggested we go for a walk outside during lunch to boost our mood. You know, sometimes a little sunshine can really brighten even the most pessimistic person's day.</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>saturnine — 침울한, 불만스러운; boost — 향상시키다, 증진시키다</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr"/>
+      <c r="T5" s="9" t="inlineStr"/>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V5" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W5" s="9" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="X5" s="9" t="inlineStr">
+        <is>
+          <t>퀴즈, 시험</t>
+        </is>
+      </c>
+      <c r="Y5" s="9" t="inlineStr">
+        <is>
+          <t>더블린 극장주 Daly가 무의미한 단어를 낙서하면 하루 만에 유행어로 만든 일화에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-12
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y5"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1119,6 +1119,123 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>blandishment</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did the salesman use a lot of blandishments to try to get you to buy that expensive phone? Yeah, he kept saying nice things about the features and offering me discounts. Don't fall for it—those are just tactics to persuade you to spend more money than you planned.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>blandishment — 설득하기 위한 달콤한 말이나 행동; persuade — 설득하다</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R6" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S6" s="9" t="inlineStr"/>
+      <c r="T6" s="9" t="inlineStr"/>
+      <c r="U6" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V6" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W6" s="9" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="X6" s="9" t="inlineStr">
+        <is>
+          <t>공황, 극도의 공포</t>
+        </is>
+      </c>
+      <c r="Y6" s="9" t="inlineStr">
+        <is>
+          <t>목신 판(Pan)이 갑자기 나타나 공포를 일으킨다는 신화에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-13
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Y7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1236,6 +1236,123 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>hale</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>My grandfather is still hale and hearty at ninety years old. He stays active every day, exercises regularly, and maintains a positive outlook on life. His doctor says he's in exceptional health. That's why we always say he's doing great despite his age.</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>hale — 건강한; exceptional — 뛰어난, 특별한</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R7" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="inlineStr"/>
+      <c r="T7" s="9" t="inlineStr"/>
+      <c r="U7" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V7" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W7" s="9" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="X7" s="9" t="inlineStr">
+        <is>
+          <t>전략</t>
+        </is>
+      </c>
+      <c r="Y7" s="9" t="inlineStr">
+        <is>
+          <t>stratos(군대) + agein(이끌다) → 장군의 기술</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-14
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y7"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1353,6 +1353,123 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: A Tale of Two Cities</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Hey, have you heard about BBC Learning English? They've got this amazing classic story called 'A Tale of Two Cities' that teaches you fifteen different ways to use the word 'time'. It's perfect if you want to improve your English while enjoying a great story. You can subscribe to their newsletter or check out their website to find it.</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>subscribe — 구독하다; classic — 고전의, 클래식한</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R8" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S8" s="9" t="inlineStr"/>
+      <c r="T8" s="9" t="inlineStr"/>
+      <c r="U8" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V8" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W8" s="9" t="inlineStr">
+        <is>
+          <t>focus</t>
+        </is>
+      </c>
+      <c r="X8" s="9" t="inlineStr">
+        <is>
+          <t>초점, 집중</t>
+        </is>
+      </c>
+      <c r="Y8" s="9" t="inlineStr">
+        <is>
+          <t>로마 가정의 화덕이 집의 중심이었던 데서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-15
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y8"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1470,6 +1470,123 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>의무·충고 조동사</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: should / ought to / had better</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: A Tale of Two Cities</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'A Tale of Two Cities,' and we'll focus on 15 different ways to use the word 'time.' You'll pick up useful vocabulary while enjoying this famous English novel. Make sure to subscribe to our newsletter so you don't miss future lessons!</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>classic — 고전적인, 유명한; focus on — ~에 집중하다, 초점을 맞추다</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S9" s="9" t="inlineStr"/>
+      <c r="T9" s="9" t="inlineStr"/>
+      <c r="U9" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V9" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W9" s="9" t="inlineStr">
+        <is>
+          <t>invest</t>
+        </is>
+      </c>
+      <c r="X9" s="9" t="inlineStr">
+        <is>
+          <t>투자하다</t>
+        </is>
+      </c>
+      <c r="Y9" s="9" t="inlineStr">
+        <is>
+          <t>중세에 왕이 신하에게 땅을 수여할 때 옷(vestis)을 입혀 권한 부여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-16
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Y10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1587,6 +1587,123 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>gamut</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you check out that new restaurant downtown? Their menu really runs the gamut—they've got everything from traditional Korean dishes to modern fusion cuisine. It's great because there's something for everyone, and the prices range from budget-friendly to premium options too.</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>runs the gamut — 다양한 범위를 포괄하다; fusion — 퓨전, 혼합</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R10" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S10" s="9" t="inlineStr"/>
+      <c r="T10" s="9" t="inlineStr"/>
+      <c r="U10" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V10" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W10" s="9" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="X10" s="9" t="inlineStr">
+        <is>
+          <t>위험, 위험을 감수하다</t>
+        </is>
+      </c>
+      <c r="Y10" s="9" t="inlineStr">
+        <is>
+          <t>항해 중 암초 근처를 항행하는 위험에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-17
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y10"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1704,6 +1704,123 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: A Tale of Two Cities</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore how the word 'time' is used in different ways. In classic stories like A Tale of Two Cities, you'll notice characters often refer to time when describing important moments. Learning these 15 different uses of 'time' will really help you understand English better and communicate more naturally in everyday conversations.</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>refer to — ~을 언급하다, 지칭하다; communicate — 소통하다, 전달하다</t>
+        </is>
+      </c>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R11" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S11" s="9" t="inlineStr"/>
+      <c r="T11" s="9" t="inlineStr"/>
+      <c r="U11" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V11" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W11" s="9" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="X11" s="9" t="inlineStr">
+        <is>
+          <t>예산</t>
+        </is>
+      </c>
+      <c r="Y11" s="9" t="inlineStr">
+        <is>
+          <t>재무장관이 예산서를 담은 가죽 가방(bougette)을 들고 의회에 출석한 데서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-18
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1821,6 +1821,123 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>동명사 vs 부정사</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Gerunds vs Infinitives</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: A Tale of Two Cities</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story called A Tale of Two Cities, and while we read it, you'll discover fifteen different ways English speakers use the word 'time'. Learning these expressions will really help you communicate more naturally in everyday situations and at work. So stick with us, and by the time we finish, you'll feel much more confident using 'time' in real conversations.</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>explore — 탐험하다, 알아보다; communicate — 소통하다, 의사소통하다</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R12" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S12" s="9" t="inlineStr"/>
+      <c r="T12" s="9" t="inlineStr"/>
+      <c r="U12" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V12" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W12" s="9" t="inlineStr">
+        <is>
+          <t>magazine</t>
+        </is>
+      </c>
+      <c r="X12" s="9" t="inlineStr">
+        <is>
+          <t>잡지, 탄창</t>
+        </is>
+      </c>
+      <c r="Y12" s="9" t="inlineStr">
+        <is>
+          <t>지식·정보를 저장해 두는 '창고'라는 의미로 출판물에 사용됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-19
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1938,6 +1938,123 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Phantom of the Opera</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Have you ever watched a classic story like The Phantom of the Opera? It's a great way to improve your English because you'll encounter the word 'stage' used in many different contexts. By learning these multiple uses, you can expand your vocabulary and understand how native speakers use everyday words in creative ways.</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>encounter — (마주) 접하다; expand — 확대하다, 늘리다</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R13" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S13" s="9" t="inlineStr"/>
+      <c r="T13" s="9" t="inlineStr"/>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V13" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W13" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X13" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y13" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-20
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y13"/>
+  <dimension ref="A1:Y14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2055,6 +2055,123 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>미래 표현 3가지</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Future Tenses: will / going to / present continuous</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Phantom of the Opera</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story called 'The Phantom of the Opera.' This story has been performed on stages around the world for many years. You'll learn different uses of the word 'stage' while enjoying this fascinating tale. So, let's begin our journey into this mysterious opera house!</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>stage — 무대; explore — 탐험하다, 살펴보다</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R14" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S14" s="9" t="inlineStr"/>
+      <c r="T14" s="9" t="inlineStr"/>
+      <c r="U14" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V14" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W14" s="9" t="inlineStr">
+        <is>
+          <t>serendipity</t>
+        </is>
+      </c>
+      <c r="X14" s="9" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운</t>
+        </is>
+      </c>
+      <c r="Y14" s="9" t="inlineStr">
+        <is>
+          <t>세 왕자가 우연히 훌륭한 발견을 하는 동화에서 Horace Walpole이 만든 단어</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-21
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2172,6 +2172,123 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>assiduous</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>Sarah's been really assiduous about protecting the local nature reserve. She works on it every single day, paying close attention to every detail. Her dedication has actually made a huge difference—they've saved so much wildlife habitat from being developed. That kind of sustained effort is what really gets things done.</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>assiduous — 성실하고 열심인, 세심한 주의를 기울이는; sustained — 지속되는, 계속되는</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R15" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S15" s="9" t="inlineStr"/>
+      <c r="T15" s="9" t="inlineStr"/>
+      <c r="U15" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V15" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W15" s="9" t="inlineStr">
+        <is>
+          <t>berserk</t>
+        </is>
+      </c>
+      <c r="X15" s="9" t="inlineStr">
+        <is>
+          <t>극도로 흥분한, 폭주하는</t>
+        </is>
+      </c>
+      <c r="Y15" s="9" t="inlineStr">
+        <is>
+          <t>전투에서 곰 가죽을 입고 광분하던 바이킹 전사에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-22
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:Y16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2289,6 +2289,123 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Phantom of the Opera</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story called The Phantom of the Opera. You'll learn eleven different uses of the word 'stage' while enjoying this fascinating tale. The story takes place in a grand theatre where mystery and drama unfold on stage every single night.</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>stage — 무대, 단계; classic — 고전적인, 명작의</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R16" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S16" s="9" t="inlineStr"/>
+      <c r="T16" s="9" t="inlineStr"/>
+      <c r="U16" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V16" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W16" s="9" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="X16" s="9" t="inlineStr">
+        <is>
+          <t>불매운동, 거부하다</t>
+        </is>
+      </c>
+      <c r="Y16" s="9" t="inlineStr">
+        <is>
+          <t>1880년 소작인들이 Boycott을 집단 거부한 사건에서 단어화</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-23
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y16"/>
+  <dimension ref="A1:Y17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2406,6 +2406,123 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>quail</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>You know, when I had to present my project in front of the whole department, I really quailed at the thought of it. My manager noticed I seemed nervous, so she gave me some confidence tips. By the time the presentation came around, I didn't quail anymore—I actually did pretty well!</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>quail — 두려워하다, 공포를 드러내다; presentation — 발표, 프레젠테이션</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S17" s="9" t="inlineStr"/>
+      <c r="T17" s="9" t="inlineStr"/>
+      <c r="U17" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V17" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W17" s="9" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="X17" s="9" t="inlineStr">
+        <is>
+          <t>멘토, 스승</t>
+        </is>
+      </c>
+      <c r="Y17" s="9" t="inlineStr">
+        <is>
+          <t>오디세우스가 트로이 전쟁 중 아들 텔레마코스 교육을 맡긴 현자의 이름에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-24
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2523,6 +2523,123 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Phantom of the Opera</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story about the Phantom of the Opera. This fascinating tale teaches us how the word 'stage' has many different meanings in English. Whether you're talking about a theatre stage or a stage of development in a project, understanding these uses will definitely enhance your English skills.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>enhance — 향상시키다, 강화하다; fascinating — 매력적인, 매혹하는</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R18" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S18" s="9" t="inlineStr"/>
+      <c r="T18" s="9" t="inlineStr"/>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V18" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="X18" s="9" t="inlineStr">
+        <is>
+          <t>경쟁자</t>
+        </is>
+      </c>
+      <c r="Y18" s="9" t="inlineStr">
+        <is>
+          <t>같은 강(rivus) 물을 사용하는 이웃 사이의 경쟁 관계에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-25
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Y19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2640,6 +2640,123 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Phantom of the Opera</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring The Phantom of the Opera, a classic story that uses the word 'stage' in many different ways. You'll learn how 'stage' can mean a platform where actors perform, but also a level or period in a process. By the end of this lesson, you'll understand all eleven uses of this versatile word.</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>versatile — 다양한 용도로 쓸 수 있는; explore — 탐험하다, 탐구하다</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S19" s="9" t="inlineStr"/>
+      <c r="T19" s="9" t="inlineStr"/>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V19" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W19" s="9" t="inlineStr">
+        <is>
+          <t>travel</t>
+        </is>
+      </c>
+      <c r="X19" s="9" t="inlineStr">
+        <is>
+          <t>여행하다</t>
+        </is>
+      </c>
+      <c r="Y19" s="9" t="inlineStr">
+        <is>
+          <t>중세 여행이 고문(tripalium)처럼 고달팠던 데서 travail(고통)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-26
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y19"/>
+  <dimension ref="A1:Y20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2757,6 +2757,123 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>symbiosis</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>You know, our company's success really depends on symbiosis with our partners. We work together, support each other, and honestly, we can't really function without them. It's kind of like how fish and plants live together in an aquarium—both sides benefit. That kind of partnership is what keeps our business strong.</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>symbiosis — 상생, 상호 의존 관계; function — 기능하다, 작동하다</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R20" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S20" s="9" t="inlineStr"/>
+      <c r="T20" s="9" t="inlineStr"/>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W20" s="9" t="inlineStr">
+        <is>
+          <t>enthusiasm</t>
+        </is>
+      </c>
+      <c r="X20" s="9" t="inlineStr">
+        <is>
+          <t>열정, 열의</t>
+        </is>
+      </c>
+      <c r="Y20" s="9" t="inlineStr">
+        <is>
+          <t>en(안에) + theos(신) → 신에게 감화받은 열정 상태</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-27
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:Y21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2874,6 +2874,123 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Romeo and Juliet</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring Shakespeare's Romeo and Juliet through the word 'cross'. This classic story shows us 13 different ways to use 'cross' in English. You'll discover how this simple word appears in everyday conversations and literature. It's a fun way to expand your vocabulary while enjoying a timeless love story.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확대하다, 늘리다; timeless — 영원한, 시대를 초월한</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R21" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S21" s="9" t="inlineStr"/>
+      <c r="T21" s="9" t="inlineStr"/>
+      <c r="U21" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V21" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W21" s="9" t="inlineStr">
+        <is>
+          <t>lucid</t>
+        </is>
+      </c>
+      <c r="X21" s="9" t="inlineStr">
+        <is>
+          <t>명확한, 이해하기 쉬운</t>
+        </is>
+      </c>
+      <c r="Y21" s="9" t="inlineStr">
+        <is>
+          <t>lux(빛)과 동근 → 명확하고 투명한 사고</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-28
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:Y22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2991,6 +2991,123 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Romeo and Juliet</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Today, we're looking at the classic story of Romeo and Juliet, and you'll discover 13 different uses of the word 'cross'. This is a great way to expand your vocabulary while enjoying one of Shakespeare's most famous works. You can find all our learning materials on the BBC Learning English website, and don't forget to subscribe to our newsletter for more content like this.</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확대하다, 늘리다; subscribe — 구독하다</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R22" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S22" s="9" t="inlineStr"/>
+      <c r="T22" s="9" t="inlineStr"/>
+      <c r="U22" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V22" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W22" s="9" t="inlineStr">
+        <is>
+          <t>colleague</t>
+        </is>
+      </c>
+      <c r="X22" s="9" t="inlineStr">
+        <is>
+          <t>동료</t>
+        </is>
+      </c>
+      <c r="Y22" s="9" t="inlineStr">
+        <is>
+          <t>col(함께) + legare(선택하다/보내다) → 같이 선발된 동료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-29
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:Y23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3108,6 +3108,123 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>umami</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>So I tried this new restaurant last night, and honestly, their dishes had amazing umami flavor. You know, that rich, savory taste you get from things like aged cheese and mushrooms? The chef told me she uses soy sauce and tomatoes as her secret ingredients to enhance the umami in everything. It's becoming a real game-changer in modern cooking.</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>umami — 우마미(감칠맛, 진하고 고소한 맛); enhance — 향상시키다, 돋보이게 하다</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R23" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S23" s="9" t="inlineStr"/>
+      <c r="T23" s="9" t="inlineStr"/>
+      <c r="U23" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V23" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W23" s="9" t="inlineStr">
+        <is>
+          <t>quarantine</t>
+        </is>
+      </c>
+      <c r="X23" s="9" t="inlineStr">
+        <is>
+          <t>격리, 검역</t>
+        </is>
+      </c>
+      <c r="Y23" s="9" t="inlineStr">
+        <is>
+          <t>14세기 흑사병 때 선박을 40일간 격리한 베네치아 방역 정책에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-06-30
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y23"/>
+  <dimension ref="A1:Y24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3225,6 +3225,123 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>bereft</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>After the company lost its main client, they felt completely bereft of resources to continue the project. The team was bereft of motivation and ideas. However, the manager decided to pivot and look for new opportunities instead of giving up.</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>bereft — ~이 없는, 박탈당한; pivot — 방향을 바꾸다, 전환하다</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R24" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S24" s="9" t="inlineStr"/>
+      <c r="T24" s="9" t="inlineStr"/>
+      <c r="U24" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V24" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W24" s="9" t="inlineStr">
+        <is>
+          <t>clue</t>
+        </is>
+      </c>
+      <c r="X24" s="9" t="inlineStr">
+        <is>
+          <t>단서, 실마리</t>
+        </is>
+      </c>
+      <c r="Y24" s="9" t="inlineStr">
+        <is>
+          <t>그리스 신화에서 테세우스가 미로를 탈출할 때 아리아드네의 실(clew)에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-01
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y24"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3342,6 +3342,123 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>nabob</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>You know, those tech company nabobs always meet at fancy restaurants to discuss business deals. They're so wealthy and powerful that everyone wants to listen to what they say. It's pretty interesting how much influence these important people have in the corporate world.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>nabob — 거물, 부자 권력가; influence — 영향력, 영향을 미치다</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P25" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R25" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S25" s="9" t="inlineStr"/>
+      <c r="T25" s="9" t="inlineStr"/>
+      <c r="U25" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V25" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W25" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X25" s="9" t="inlineStr">
+        <is>
+          <t>급여</t>
+        </is>
+      </c>
+      <c r="Y25" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사의 소금 급여에서. '소금값 못하는 사람'이라는 표현도 여기서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-02
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y25"/>
+  <dimension ref="A1:Y26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3459,6 +3459,123 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>현재완료 vs 단순과거</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Present Perfect vs Simple Past</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>sagacious</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>Our new manager has really impressed everyone with her sagacious decisions. She doesn't just solve problems—she understands what's really going on beneath the surface. That's why people respect her judgment so much. When you need advice on a tricky situation, she's the person to talk to.</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>sagacious — 현명한, 통찰력 있는; beneath the surface — 표면 아래에, 겉으로는 보이지 않는</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P26" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q26" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R26" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S26" s="9" t="inlineStr"/>
+      <c r="T26" s="9" t="inlineStr"/>
+      <c r="U26" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V26" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W26" s="9" t="inlineStr">
+        <is>
+          <t>sincere</t>
+        </is>
+      </c>
+      <c r="X26" s="9" t="inlineStr">
+        <is>
+          <t>진실한, 진심 어린</t>
+        </is>
+      </c>
+      <c r="Y26" s="9" t="inlineStr">
+        <is>
+          <t>로마 조각가가 결함을 밀랍으로 숨겼는데, 최고 작품은 밀랍 없이(sine cera) 완성됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-03
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y26"/>
+  <dimension ref="A1:Y27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3576,6 +3576,123 @@
         </is>
       </c>
     </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'The Red Shoes,' which teaches us different ways to use the word 'wear.' You'll discover thirteen different meanings of this common verb through an engaging narrative. It's a fantastic resource if you want to expand your vocabulary and improve your listening skills at the same time.</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확장하다, 늘리다; resource — 자료, 도움이 되는 것</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q27" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R27" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S27" s="9" t="inlineStr"/>
+      <c r="T27" s="9" t="inlineStr"/>
+      <c r="U27" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V27" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W27" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X27" s="9" t="inlineStr">
+        <is>
+          <t>급여, 봉급</t>
+        </is>
+      </c>
+      <c r="Y27" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사는 소금(sal)으로 급여를 받았음. salt와 같은 어근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-04
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y27"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3693,6 +3693,123 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'The Red Shoes,' which explores different ways we use the word 'wear' in English. You'll discover thirteen different meanings of this common verb through the narrative. It's a great way to expand your vocabulary and understand how one word can have multiple uses in everyday conversation.</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>explores — 탐구하다, 살펴보다; vocabulary — 어휘, 단어</t>
+        </is>
+      </c>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N28" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O28" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P28" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q28" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R28" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S28" s="9" t="inlineStr"/>
+      <c r="T28" s="9" t="inlineStr"/>
+      <c r="U28" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V28" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W28" s="9" t="inlineStr">
+        <is>
+          <t>muscle</t>
+        </is>
+      </c>
+      <c r="X28" s="9" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="Y28" s="9" t="inlineStr">
+        <is>
+          <t>팔을 구부릴 때 근육이 움직이는 모습이 쥐처럼 보인다 하여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-05
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y28"/>
+  <dimension ref="A1:Y29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3810,6 +3810,123 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'The Red Shoes,' which teaches us about the word 'wear' and its different meanings. You'll discover how 'wear' can mean to have clothes on your body, but also to gradually damage or exhaust something over time. By learning these 13 uses of 'wear,' you'll be able to express yourself more naturally in English conversations.</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>wear — 입다, 차다; 닳다, 지치다; exhaust — 지치게 하다, 소진하다</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N29" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O29" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P29" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R29" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S29" s="9" t="inlineStr"/>
+      <c r="T29" s="9" t="inlineStr"/>
+      <c r="U29" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V29" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W29" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X29" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y29" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가(candida)를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-06
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y29"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3927,6 +3927,123 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic story called 'The Red Shoes' and discover thirteen different ways to use the word 'wear'. This story teaches us about how our choices and fashion can really impact our lives. If you subscribe to our newsletter, you'll get weekly tips to help you improve your English skills.</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>subscribe — 구독하다; impact — 영향을 미치다</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P30" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q30" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R30" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S30" s="9" t="inlineStr"/>
+      <c r="T30" s="9" t="inlineStr"/>
+      <c r="U30" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V30" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W30" s="9" t="inlineStr">
+        <is>
+          <t>disaster</t>
+        </is>
+      </c>
+      <c r="X30" s="9" t="inlineStr">
+        <is>
+          <t>재앙, 참사</t>
+        </is>
+      </c>
+      <c r="Y30" s="9" t="inlineStr">
+        <is>
+          <t>별의 위치가 나쁘면 재앙이 온다는 점성술 믿음에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-07
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y30"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4044,6 +4044,123 @@
         </is>
       </c>
     </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'The Red Shoes' and focusing on different uses of the word 'wear'. You'll discover how this word appears in everyday conversations and storytelling. It's a great way to expand your vocabulary while enjoying an engaging tale.</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확장하다, 늘리다; engaging — 흥미로운, 매력적인</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P31" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q31" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R31" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S31" s="9" t="inlineStr"/>
+      <c r="T31" s="9" t="inlineStr"/>
+      <c r="U31" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V31" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W31" s="9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="X31" s="9" t="inlineStr">
+        <is>
+          <t>회사, 동료</t>
+        </is>
+      </c>
+      <c r="Y31" s="9" t="inlineStr">
+        <is>
+          <t>같이 빵을 나눠 먹는 동료에서 유래. companion(동료)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-08
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:Y32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4161,6 +4161,123 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>Have you ever heard of 'The Red Shoes'? It's a classic fairy tale about a girl who receives a special pair of shoes. Once she starts wearing them, she can't stop dancing! Today, we're going to explore thirteen different ways to use the word 'wear' while enjoying this timeless story.</t>
+        </is>
+      </c>
+      <c r="K32" s="9" t="inlineStr">
+        <is>
+          <t>wear — 입다, 신다, 쓰다 (옷이나 신발을 몸에 걸치다); classic — 고전적인, 클래식한 (오래되고 뛰어난)</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P32" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q32" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R32" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S32" s="9" t="inlineStr"/>
+      <c r="T32" s="9" t="inlineStr"/>
+      <c r="U32" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V32" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W32" s="9" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="X32" s="9" t="inlineStr">
+        <is>
+          <t>계산하다</t>
+        </is>
+      </c>
+      <c r="Y32" s="9" t="inlineStr">
+        <is>
+          <t>로마인이 주판 대신 조약돌(calculus)로 계산했음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-09
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:Y33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4278,6 +4278,123 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>의무·충고 조동사</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: should / ought to / had better</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I33" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Red Shoes</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring a classic story called 'The Red Shoes' and learning different ways to use the word 'wear'. You'll discover thirteen different meanings, from wearing clothes to wearing out your patience. This podcast helps you understand how native speakers use everyday vocabulary in real situations.</t>
+        </is>
+      </c>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>wear — (입다, 착용하다) 또는 (닳다, 소진하다); explore — (탐색하다, 살펴보다)</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N33" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q33" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R33" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S33" s="9" t="inlineStr"/>
+      <c r="T33" s="9" t="inlineStr"/>
+      <c r="U33" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V33" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W33" s="9" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="X33" s="9" t="inlineStr">
+        <is>
+          <t>마감 기한</t>
+        </is>
+      </c>
+      <c r="Y33" s="9" t="inlineStr">
+        <is>
+          <t>남북전쟁 포로수용소에서 그 선을 넘으면 사살한다는 경계선에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-10
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y33"/>
+  <dimension ref="A1:Y34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4395,6 +4395,123 @@
         </is>
       </c>
     </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>effulgence</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>Last night, we finally finished decorating the office lobby with all those new lights. When we turned them on, the whole space just lit up with this amazing effulgence—it was like stepping into Times Square! The clients who came in this morning were really impressed by the sudden brilliance. Sometimes the simplest decorations can completely transform how people feel when they walk through the door.</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
+        <is>
+          <t>effulgence — 광채, 찬란함; transform — 변화시키다, 변모시키다</t>
+        </is>
+      </c>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N34" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P34" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q34" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R34" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S34" s="9" t="inlineStr"/>
+      <c r="T34" s="9" t="inlineStr"/>
+      <c r="U34" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V34" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W34" s="9" t="inlineStr">
+        <is>
+          <t>bankrupt</t>
+        </is>
+      </c>
+      <c r="X34" s="9" t="inlineStr">
+        <is>
+          <t>파산한</t>
+        </is>
+      </c>
+      <c r="Y34" s="9" t="inlineStr">
+        <is>
+          <t>중세 환전상이 파산하면 거래 탁자(banca)를 부수는 관습에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-11
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y34"/>
+  <dimension ref="A1:Y35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4512,6 +4512,123 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Oliver Twist</t>
+        </is>
+      </c>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story, Oliver Twist, and we'll explore seven different uses of the word 'light'. This is a great way to expand your vocabulary in just five minutes. You can listen to this story anytime, anywhere, and follow along on our website. Don't forget to check out our other popular podcasts like 6 Minute English if you want to keep learning!</t>
+        </is>
+      </c>
+      <c r="K35" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확장하다, 늘리다; classic — 고전의, 클래식한</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N35" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P35" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q35" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R35" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S35" s="9" t="inlineStr"/>
+      <c r="T35" s="9" t="inlineStr"/>
+      <c r="U35" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V35" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W35" s="9" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="X35" s="9" t="inlineStr">
+        <is>
+          <t>퀴즈, 시험</t>
+        </is>
+      </c>
+      <c r="Y35" s="9" t="inlineStr">
+        <is>
+          <t>더블린 극장주 Daly가 무의미한 단어를 낙서하면 하루 만에 유행어로 만든 일화에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-12
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y35"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4629,6 +4629,123 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>동명사 vs 부정사</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Gerunds vs Infinitives</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Oliver Twist</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>Hey, have you ever read Oliver Twist? It's a classic story that can really help you improve your English. In just five minutes, you'll learn seven different uses of the word 'light' while enjoying this amazing tale. It's a fantastic way to boost your vocabulary naturally.</t>
+        </is>
+      </c>
+      <c r="K36" s="9" t="inlineStr">
+        <is>
+          <t>classic — 고전의; boost — 향상시키다</t>
+        </is>
+      </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M36" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N36" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P36" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q36" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R36" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S36" s="9" t="inlineStr"/>
+      <c r="T36" s="9" t="inlineStr"/>
+      <c r="U36" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V36" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W36" s="9" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="X36" s="9" t="inlineStr">
+        <is>
+          <t>공황, 극도의 공포</t>
+        </is>
+      </c>
+      <c r="Y36" s="9" t="inlineStr">
+        <is>
+          <t>목신 판(Pan)이 갑자기 나타나 공포를 일으킨다는 신화에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-13
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y36"/>
+  <dimension ref="A1:Y37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4746,6 +4746,123 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Oliver Twist</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring a classic story, Oliver Twist, and learning different uses of the word 'light'. The BBC Learning English team has created this five-minute lesson to help you understand how 'light' works in everyday English. You can find more stories and podcasts on their website, so don't hesitate to check them out!</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>explore — 탐구하다, 살펴보다; hesitate — 주저하다, 망설이다</t>
+        </is>
+      </c>
+      <c r="L37" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N37" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P37" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q37" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R37" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S37" s="9" t="inlineStr"/>
+      <c r="T37" s="9" t="inlineStr"/>
+      <c r="U37" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V37" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W37" s="9" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="X37" s="9" t="inlineStr">
+        <is>
+          <t>전략</t>
+        </is>
+      </c>
+      <c r="Y37" s="9" t="inlineStr">
+        <is>
+          <t>stratos(군대) + agein(이끌다) → 장군의 기술</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-14
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y37"/>
+  <dimension ref="A1:Y38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4863,6 +4863,123 @@
         </is>
       </c>
     </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>미래 표현 3가지</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Future Tenses: will / going to / present continuous</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Oliver Twist</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>Hey, have you ever read Oliver Twist? It's a classic story that really sheds light on life in Victorian England. The BBC Learning English team created a five-minute version that teaches you seven different uses of the word 'light.' It's a brilliant way to improve your vocabulary while enjoying a famous novel.</t>
+        </is>
+      </c>
+      <c r="K38" s="9" t="inlineStr">
+        <is>
+          <t>shed light on — ~을 명확히 하다, 설명하다; brilliant — 훌륭한, 멋진</t>
+        </is>
+      </c>
+      <c r="L38" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N38" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P38" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q38" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R38" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S38" s="9" t="inlineStr"/>
+      <c r="T38" s="9" t="inlineStr"/>
+      <c r="U38" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V38" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W38" s="9" t="inlineStr">
+        <is>
+          <t>focus</t>
+        </is>
+      </c>
+      <c r="X38" s="9" t="inlineStr">
+        <is>
+          <t>초점, 집중</t>
+        </is>
+      </c>
+      <c r="Y38" s="9" t="inlineStr">
+        <is>
+          <t>로마 가정의 화덕이 집의 중심이었던 데서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-15
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y38"/>
+  <dimension ref="A1:Y39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4980,6 +4980,123 @@
         </is>
       </c>
     </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>loquacious</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>My new colleague is really loquacious—she talks constantly during meetings and uses way too many words to explain simple things. It's kind of exhausting, honestly. I think she means well, but she should probably work on being more concise with her presentations.</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>loquacious — 말을 많이 하는, 수다스러운; concise — 간결한, 간단한</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P39" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R39" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S39" s="9" t="inlineStr"/>
+      <c r="T39" s="9" t="inlineStr"/>
+      <c r="U39" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V39" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W39" s="9" t="inlineStr">
+        <is>
+          <t>invest</t>
+        </is>
+      </c>
+      <c r="X39" s="9" t="inlineStr">
+        <is>
+          <t>투자하다</t>
+        </is>
+      </c>
+      <c r="Y39" s="9" t="inlineStr">
+        <is>
+          <t>중세에 왕이 신하에게 땅을 수여할 때 옷(vestis)을 입혀 권한 부여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-16
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y39"/>
+  <dimension ref="A1:Y40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5097,6 +5097,123 @@
         </is>
       </c>
     </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>bibelot</t>
+        </is>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>So my grandmother just opened a small antique shop, and she's been collecting bibelots for years—you know, little decorative objects like ceramic figurines and glass sculptures. She spent the whole weekend organizing everything on shelves and in display cases. The shop looks amazing, but honestly, I had no idea there were so many different words for trinkets in English!</t>
+        </is>
+      </c>
+      <c r="K40" s="9" t="inlineStr">
+        <is>
+          <t>bibelot — 소품, 장식용 물건; organize — 정리하다, 정렬하다</t>
+        </is>
+      </c>
+      <c r="L40" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N40" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O40" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P40" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q40" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R40" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S40" s="9" t="inlineStr"/>
+      <c r="T40" s="9" t="inlineStr"/>
+      <c r="U40" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V40" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W40" s="9" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="X40" s="9" t="inlineStr">
+        <is>
+          <t>위험, 위험을 감수하다</t>
+        </is>
+      </c>
+      <c r="Y40" s="9" t="inlineStr">
+        <is>
+          <t>항해 중 암초 근처를 항행하는 위험에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-17
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:Y41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5214,6 +5214,123 @@
         </is>
       </c>
     </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>obdurate</t>
+        </is>
+      </c>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>Our team tried to convince the manager to adopt new software, but he was pretty obdurate about keeping the old system. No matter what data we showed him, he just wouldn't budge. Finally, we had to escalate the issue to leadership. Sometimes you have to accept that certain people are just resistant to change.</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
+        <is>
+          <t>obdurate — 완고한, 설득에 응하지 않는; escalate — 상황을 높은 수준으로 올리다, 확대하다</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N41" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O41" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P41" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q41" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R41" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S41" s="9" t="inlineStr"/>
+      <c r="T41" s="9" t="inlineStr"/>
+      <c r="U41" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V41" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W41" s="9" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="X41" s="9" t="inlineStr">
+        <is>
+          <t>예산</t>
+        </is>
+      </c>
+      <c r="Y41" s="9" t="inlineStr">
+        <is>
+          <t>재무장관이 예산서를 담은 가죽 가방(bougette)을 들고 의회에 출석한 데서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-18
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y41"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5331,6 +5331,123 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: David Copperfield</t>
+        </is>
+      </c>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>Hey, have you ever read David Copperfield? It's a classic novel that can really help you improve your English. The BBC Learning English team has created a special five-minute story using different meanings of the word 'take'. It's a great way to learn vocabulary while enjoying a famous story.</t>
+        </is>
+      </c>
+      <c r="K42" s="9" t="inlineStr">
+        <is>
+          <t>classic — 고전의, 명작의; improve — 향상시키다, 개선하다</t>
+        </is>
+      </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P42" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q42" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R42" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S42" s="9" t="inlineStr"/>
+      <c r="T42" s="9" t="inlineStr"/>
+      <c r="U42" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V42" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W42" s="9" t="inlineStr">
+        <is>
+          <t>magazine</t>
+        </is>
+      </c>
+      <c r="X42" s="9" t="inlineStr">
+        <is>
+          <t>잡지, 탄창</t>
+        </is>
+      </c>
+      <c r="Y42" s="9" t="inlineStr">
+        <is>
+          <t>지식·정보를 저장해 두는 '창고'라는 의미로 출판물에 사용됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-19
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y42"/>
+  <dimension ref="A1:Y43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5448,6 +5448,123 @@
         </is>
       </c>
     </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: David Copperfield</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic English story called David Copperfield and learn different ways to use the verb 'take'. Understanding phrasal verbs with 'take' is essential for everyday conversation. So let's dive in and take a closer look at these useful expressions that you'll encounter in business and daily life.</t>
+        </is>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>essential — 필수적인; phrasal verbs — 구동사</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P43" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q43" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R43" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S43" s="9" t="inlineStr"/>
+      <c r="T43" s="9" t="inlineStr"/>
+      <c r="U43" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V43" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W43" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X43" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y43" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-20
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y43"/>
+  <dimension ref="A1:Y44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5565,6 +5565,123 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>raffish</t>
+        </is>
+      </c>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>You know, my boss has this raffish style that shouldn't work, but somehow it does. He shows up in casual clothes, tells jokes in meetings, and challenges the company rules. At first, I thought he was unprofessional, but his unconventional charm actually motivates the whole team. We respect him because he's careless about formality but serious about results.</t>
+        </is>
+      </c>
+      <c r="K44" s="9" t="inlineStr">
+        <is>
+          <t>raffish — 매력적인 비정통적인 태도; unconventional — 관습적이지 않은</t>
+        </is>
+      </c>
+      <c r="L44" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M44" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N44" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P44" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q44" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R44" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S44" s="9" t="inlineStr"/>
+      <c r="T44" s="9" t="inlineStr"/>
+      <c r="U44" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V44" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W44" s="9" t="inlineStr">
+        <is>
+          <t>serendipity</t>
+        </is>
+      </c>
+      <c r="X44" s="9" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운</t>
+        </is>
+      </c>
+      <c r="Y44" s="9" t="inlineStr">
+        <is>
+          <t>세 왕자가 우연히 훌륭한 발견을 하는 동화에서 Horace Walpole이 만든 단어</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-21
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y44"/>
+  <dimension ref="A1:Y45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5682,6 +5682,123 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>dog days</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>Hey, have you noticed how unproductive everyone gets during the dog days of summer? Yeah, it's that really hot period from July through early September when it's hard to focus at work. People just don't have the energy to tackle serious projects. That's why many companies actually slow down their schedules during this time.</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>dog days — 한여름의 가장 더운 시기, 무기력한 시기; unproductive — 생산성이 낮은, 비효율적인</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O45" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P45" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q45" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R45" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S45" s="9" t="inlineStr"/>
+      <c r="T45" s="9" t="inlineStr"/>
+      <c r="U45" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V45" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W45" s="9" t="inlineStr">
+        <is>
+          <t>berserk</t>
+        </is>
+      </c>
+      <c r="X45" s="9" t="inlineStr">
+        <is>
+          <t>극도로 흥분한, 폭주하는</t>
+        </is>
+      </c>
+      <c r="Y45" s="9" t="inlineStr">
+        <is>
+          <t>전투에서 곰 가죽을 입고 광분하던 바이킹 전사에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-22
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y45"/>
+  <dimension ref="A1:Y46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5799,6 +5799,123 @@
         </is>
       </c>
     </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: David Copperfield</t>
+        </is>
+      </c>
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you know that the verb 'take' has over 13 different meanings in English? It's really useful for daily conversations. In this BBC Learning English story about David Copperfield, you'll discover how native speakers actually use 'take' in real situations. It's a classic tale that'll help you improve your English naturally in just five minutes.</t>
+        </is>
+      </c>
+      <c r="K46" s="9" t="inlineStr">
+        <is>
+          <t>native speakers — 원어민; discover — 발견하다</t>
+        </is>
+      </c>
+      <c r="L46" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N46" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O46" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P46" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q46" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R46" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S46" s="9" t="inlineStr"/>
+      <c r="T46" s="9" t="inlineStr"/>
+      <c r="U46" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V46" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W46" s="9" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="X46" s="9" t="inlineStr">
+        <is>
+          <t>불매운동, 거부하다</t>
+        </is>
+      </c>
+      <c r="Y46" s="9" t="inlineStr">
+        <is>
+          <t>1880년 소작인들이 Boycott을 집단 거부한 사건에서 단어화</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-23
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y46"/>
+  <dimension ref="A1:Y47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5916,6 +5916,123 @@
         </is>
       </c>
     </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>maverick</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>You know, Steve Jobs was kind of a maverick in the tech industry. He didn't follow what other companies were doing—he just did his own thing. That's why Apple became so innovative and successful. Being a maverick means you're willing to take risks and challenge the status quo.</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>maverick — 관례를 거부하는 사람, 독립적 인물; innovative — 혁신적인, 새로운 아이디어를 가진</t>
+        </is>
+      </c>
+      <c r="L47" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N47" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O47" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P47" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q47" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R47" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S47" s="9" t="inlineStr"/>
+      <c r="T47" s="9" t="inlineStr"/>
+      <c r="U47" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V47" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W47" s="9" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="X47" s="9" t="inlineStr">
+        <is>
+          <t>멘토, 스승</t>
+        </is>
+      </c>
+      <c r="Y47" s="9" t="inlineStr">
+        <is>
+          <t>오디세우스가 트로이 전쟁 중 아들 텔레마코스 교육을 맡긴 현자의 이름에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-24
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y47"/>
+  <dimension ref="A1:Y48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6033,6 +6033,123 @@
         </is>
       </c>
     </row>
+    <row r="48" ht="60" customHeight="1">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Dr Jekyll and Mr Hyde</t>
+        </is>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called Dr Jekyll and Mr Hyde. It's a fascinating tale about a scientist who creates a potion that transforms him into a completely different person. By studying this story, you'll learn nine different uses of the word 'sound' and improve your English listening skills in just five minutes.</t>
+        </is>
+      </c>
+      <c r="K48" s="9" t="inlineStr">
+        <is>
+          <t>potion — 약물, 마법의 음료; transform — 변환하다, 변신하다</t>
+        </is>
+      </c>
+      <c r="L48" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N48" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O48" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P48" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q48" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R48" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S48" s="9" t="inlineStr"/>
+      <c r="T48" s="9" t="inlineStr"/>
+      <c r="U48" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V48" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W48" s="9" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="X48" s="9" t="inlineStr">
+        <is>
+          <t>경쟁자</t>
+        </is>
+      </c>
+      <c r="Y48" s="9" t="inlineStr">
+        <is>
+          <t>같은 강(rivus) 물을 사용하는 이웃 사이의 경쟁 관계에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-25
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Y49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6150,6 +6150,123 @@
         </is>
       </c>
     </row>
+    <row r="49" ht="60" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Dr Jekyll and Mr Hyde</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>Dr Jekyll and Mr Hyde is a classic story about a scientist who discovers a potion that transforms him into an evil version of himself. The story explores how sound can reveal a character's true nature—when Mr Hyde speaks, his voice sounds menacing and dangerous. By studying this tale, you'll learn nine different uses of the word 'sound' in just five minutes.</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>transform — 변환하다, 변신하다; menacing — 위협적인, 위협을 나타내는</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O49" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P49" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q49" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R49" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S49" s="9" t="inlineStr"/>
+      <c r="T49" s="9" t="inlineStr"/>
+      <c r="U49" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V49" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W49" s="9" t="inlineStr">
+        <is>
+          <t>travel</t>
+        </is>
+      </c>
+      <c r="X49" s="9" t="inlineStr">
+        <is>
+          <t>여행하다</t>
+        </is>
+      </c>
+      <c r="Y49" s="9" t="inlineStr">
+        <is>
+          <t>중세 여행이 고문(tripalium)처럼 고달팠던 데서 travail(고통)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-26
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y49"/>
+  <dimension ref="A1:Y50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6267,6 +6267,123 @@
         </is>
       </c>
     </row>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>현재완료 vs 단순과거</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Present Perfect vs Simple Past</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>aerie</t>
+        </is>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you see that eagle documentary? The pair built their aerie on top of a cliff, and it's amazing how high up it is. They keep adding sticks and grass to maintain their nest, kind of like doing home improvements. You can really get a bird's-eye view of everything from up there.</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>aerie — (새의) 둥지, 높은 곳의 보금자리; bird's-eye view — 새가 보는 듯한 전망, 조감도</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N50" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O50" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P50" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q50" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R50" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S50" s="9" t="inlineStr"/>
+      <c r="T50" s="9" t="inlineStr"/>
+      <c r="U50" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V50" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W50" s="9" t="inlineStr">
+        <is>
+          <t>enthusiasm</t>
+        </is>
+      </c>
+      <c r="X50" s="9" t="inlineStr">
+        <is>
+          <t>열정, 열의</t>
+        </is>
+      </c>
+      <c r="Y50" s="9" t="inlineStr">
+        <is>
+          <t>en(안에) + theos(신) → 신에게 감화받은 열정 상태</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-27
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y50"/>
+  <dimension ref="A1:Y51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6384,6 +6384,123 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Dr Jekyll and Mr Hyde</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at the classic story of Dr Jekyll and Mr Hyde, which explores how one person can have two completely different personalities. The narrative really demonstrates how sound can be used to create tension and fear throughout the tale. If you want to improve your English and learn more about storytelling techniques, BBC Learning English has a free five-minute lesson that breaks down nine different uses of the word 'sound'.</t>
+        </is>
+      </c>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>narrative — 이야기, 서사; demonstrate — 보여주다, 증명하다</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N51" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O51" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P51" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q51" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R51" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S51" s="9" t="inlineStr"/>
+      <c r="T51" s="9" t="inlineStr"/>
+      <c r="U51" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V51" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W51" s="9" t="inlineStr">
+        <is>
+          <t>lucid</t>
+        </is>
+      </c>
+      <c r="X51" s="9" t="inlineStr">
+        <is>
+          <t>명확한, 이해하기 쉬운</t>
+        </is>
+      </c>
+      <c r="Y51" s="9" t="inlineStr">
+        <is>
+          <t>lux(빛)과 동근 → 명확하고 투명한 사고</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-28
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y51"/>
+  <dimension ref="A1:Y52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6501,6 +6501,123 @@
         </is>
       </c>
     </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>kludge</t>
+        </is>
+      </c>
+      <c r="J52" s="9" t="inlineStr">
+        <is>
+          <t>So my team needed to fix a bug in our system really quickly. We didn't have time for a perfect solution, so we just implemented a kludge—a temporary workaround that got things running again. It's not ideal, but it buys us time to develop something more robust later.</t>
+        </is>
+      </c>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>kludge — 임시방편, 땜질식 해결책; robust — 견고한, 튼튼한</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N52" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O52" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P52" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q52" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R52" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S52" s="9" t="inlineStr"/>
+      <c r="T52" s="9" t="inlineStr"/>
+      <c r="U52" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V52" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W52" s="9" t="inlineStr">
+        <is>
+          <t>colleague</t>
+        </is>
+      </c>
+      <c r="X52" s="9" t="inlineStr">
+        <is>
+          <t>동료</t>
+        </is>
+      </c>
+      <c r="Y52" s="9" t="inlineStr">
+        <is>
+          <t>col(함께) + legare(선택하다/보내다) → 같이 선발된 동료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-29
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y52"/>
+  <dimension ref="A1:Y53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6618,6 +6618,123 @@
         </is>
       </c>
     </row>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>inveigle</t>
+        </is>
+      </c>
+      <c r="J53" s="9" t="inlineStr">
+        <is>
+          <t>My boss tried to inveigle me into working extra hours by promising a promotion. I knew it was just a clever trick, so I politely declined. Sometimes people use deceptive tactics to get what they want, but it's important to recognize when someone is manipulating you.</t>
+        </is>
+      </c>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>inveigle — 교묘하게 속여 설득하다; manipulation — 조종, 부당한 영향</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N53" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O53" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P53" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q53" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R53" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S53" s="9" t="inlineStr"/>
+      <c r="T53" s="9" t="inlineStr"/>
+      <c r="U53" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V53" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W53" s="9" t="inlineStr">
+        <is>
+          <t>quarantine</t>
+        </is>
+      </c>
+      <c r="X53" s="9" t="inlineStr">
+        <is>
+          <t>격리, 검역</t>
+        </is>
+      </c>
+      <c r="Y53" s="9" t="inlineStr">
+        <is>
+          <t>14세기 흑사병 때 선박을 40일간 격리한 베네치아 방역 정책에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-30
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y53"/>
+  <dimension ref="A1:Y54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6735,6 +6735,123 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Dr Jekyll and Mr Hyde</t>
+        </is>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>Have you ever heard of Dr Jekyll and Mr Hyde? It's a classic story about a scientist who discovers a potion that transforms him into a completely different person. The interesting thing is how the story uses sound to show the character's inner conflict. Learning English through classic stories like this is actually a really effective method.</t>
+        </is>
+      </c>
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>potion — 약, 묘약; inner conflict — 내적 갈등</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N54" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O54" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P54" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q54" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R54" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S54" s="9" t="inlineStr"/>
+      <c r="T54" s="9" t="inlineStr"/>
+      <c r="U54" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V54" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W54" s="9" t="inlineStr">
+        <is>
+          <t>clue</t>
+        </is>
+      </c>
+      <c r="X54" s="9" t="inlineStr">
+        <is>
+          <t>단서, 실마리</t>
+        </is>
+      </c>
+      <c r="Y54" s="9" t="inlineStr">
+        <is>
+          <t>그리스 신화에서 테세우스가 미로를 탈출할 때 아리아드네의 실(clew)에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-07-31
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y54"/>
+  <dimension ref="A1:Y55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6852,6 +6852,123 @@
         </is>
       </c>
     </row>
+    <row r="55" ht="60" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>comely</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you see that article about Berlin pigeons? The writer said some of them were actually pretty comely, way more attractive than the ones in New York. It's funny how he used such an old-fashioned word to describe birds. I guess writers really do pick interesting vocabulary when they want to sound more literary.</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>comely — 아름다운, 매력적인 (구식 표현); literary — 문학적인, 문학다운</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O55" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P55" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q55" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R55" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S55" s="9" t="inlineStr"/>
+      <c r="T55" s="9" t="inlineStr"/>
+      <c r="U55" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V55" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W55" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X55" s="9" t="inlineStr">
+        <is>
+          <t>급여</t>
+        </is>
+      </c>
+      <c r="Y55" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사의 소금 급여에서. '소금값 못하는 사람'이라는 표현도 여기서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-01
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y55"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6969,6 +6969,123 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="60" customHeight="1">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="inlineStr">
+        <is>
+          <t>spindrift</t>
+        </is>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>So I went on this amazing whale-watching tour last weekend, right? The waves were pretty intense, and there was so much spindrift—you know, that spray from the waves—just hitting us constantly. My clothes were soaked, but honestly, it was an unforgettable experience. I'd definitely recommend it if you're into marine life.</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="inlineStr">
+        <is>
+          <t>spindrift — 파도에서 튀어나오는 물입자; unforgettable — 잊을 수 없는</t>
+        </is>
+      </c>
+      <c r="L56" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N56" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O56" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P56" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q56" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R56" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S56" s="9" t="inlineStr"/>
+      <c r="T56" s="9" t="inlineStr"/>
+      <c r="U56" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V56" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W56" s="9" t="inlineStr">
+        <is>
+          <t>sincere</t>
+        </is>
+      </c>
+      <c r="X56" s="9" t="inlineStr">
+        <is>
+          <t>진실한, 진심 어린</t>
+        </is>
+      </c>
+      <c r="Y56" s="9" t="inlineStr">
+        <is>
+          <t>로마 조각가가 결함을 밀랍으로 숨겼는데, 최고 작품은 밀랍 없이(sine cera) 완성됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-02
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y56"/>
+  <dimension ref="A1:Y57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7086,6 +7086,123 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>의무·충고 조동사</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: should / ought to / had better</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Frankenstein</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore Mary Shelley's classic novel, Frankenstein, and learn how the verb 'make' is used in different ways throughout the story. The monster was made from dead body parts, and Victor Frankenstein's ambition made him create this terrifying creature. Understanding these uses of 'make' will definitely make your English stronger!</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>ambition — 야망, 열망; creature — 생물, 창조물</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N57" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O57" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P57" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q57" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R57" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S57" s="9" t="inlineStr"/>
+      <c r="T57" s="9" t="inlineStr"/>
+      <c r="U57" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V57" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W57" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X57" s="9" t="inlineStr">
+        <is>
+          <t>급여, 봉급</t>
+        </is>
+      </c>
+      <c r="Y57" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사는 소금(sal)으로 급여를 받았음. salt와 같은 어근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-03
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y57"/>
+  <dimension ref="A1:Y58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7203,6 +7203,123 @@
         </is>
       </c>
     </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I58" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Frankenstein</t>
+        </is>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore the classic story of Frankenstein and learn how the verb 'make' is used in different ways. This engaging lesson will help you understand ten different meanings of 'make' in just five minutes. You can subscribe to our free newsletter to get more learning content delivered straight to your inbox every week.</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>engage — 몰두하게 하다, 참여시키다; subscribe — 구독하다, 신청하다</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N58" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O58" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P58" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q58" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R58" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S58" s="9" t="inlineStr"/>
+      <c r="T58" s="9" t="inlineStr"/>
+      <c r="U58" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V58" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W58" s="9" t="inlineStr">
+        <is>
+          <t>muscle</t>
+        </is>
+      </c>
+      <c r="X58" s="9" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="Y58" s="9" t="inlineStr">
+        <is>
+          <t>팔을 구부릴 때 근육이 움직이는 모습이 쥐처럼 보인다 하여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-04
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y58"/>
+  <dimension ref="A1:Y59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7320,6 +7320,123 @@
         </is>
       </c>
     </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I59" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Frankenstein</t>
+        </is>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at the classic story of Frankenstein, and we'll focus on different uses of the word 'make' throughout the narrative. Victor Frankenstein makes a terrible decision that changes his life forever. By studying these ten examples, you'll understand how 'make' appears in everyday English and literature.</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>narrative — 이야기, 서술; decision — 결정, 판단</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N59" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O59" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P59" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q59" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R59" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S59" s="9" t="inlineStr"/>
+      <c r="T59" s="9" t="inlineStr"/>
+      <c r="U59" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V59" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W59" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X59" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y59" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가(candida)를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-05
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y59"/>
+  <dimension ref="A1:Y60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7437,6 +7437,123 @@
         </is>
       </c>
     </row>
+    <row r="60" ht="60" customHeight="1">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>동명사 vs 부정사</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>Gerunds vs Infinitives</t>
+        </is>
+      </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="inlineStr">
+        <is>
+          <t>colloquial</t>
+        </is>
+      </c>
+      <c r="J60" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you notice how Sarah switches between formal language in her presentations and casual, colloquial style when she talks to the team? That's actually a really smart communication skill. In business, you gotta adapt your language depending on who you're talking to and what the situation is.</t>
+        </is>
+      </c>
+      <c r="K60" s="9" t="inlineStr">
+        <is>
+          <t>colloquial — 편한, 자연스러운 (말투); adapt — 적응하다, 조절하다</t>
+        </is>
+      </c>
+      <c r="L60" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N60" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O60" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P60" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q60" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R60" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S60" s="9" t="inlineStr"/>
+      <c r="T60" s="9" t="inlineStr"/>
+      <c r="U60" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V60" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W60" s="9" t="inlineStr">
+        <is>
+          <t>disaster</t>
+        </is>
+      </c>
+      <c r="X60" s="9" t="inlineStr">
+        <is>
+          <t>재앙, 참사</t>
+        </is>
+      </c>
+      <c r="Y60" s="9" t="inlineStr">
+        <is>
+          <t>별의 위치가 나쁘면 재앙이 온다는 점성술 믿음에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-07
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y60"/>
+  <dimension ref="A1:Y61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7554,6 +7554,123 @@
         </is>
       </c>
     </row>
+    <row r="61" ht="60" customHeight="1">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="inlineStr">
+        <is>
+          <t>torpor</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>You know that feeling when you're stuck indoors on a rainy day and you just can't get motivated? That's torpor—basically a state of being sluggish and inactive. Even animals experience it. Bats, for example, can enter torpor during cold snaps when they can't find insects to eat. It's like a mini-hibernation that helps them survive tough conditions.</t>
+        </is>
+      </c>
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>torpor — 무기력함, 나른함; motivated — 동기가 생긴, 의욕적인</t>
+        </is>
+      </c>
+      <c r="L61" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N61" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O61" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P61" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q61" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R61" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S61" s="9" t="inlineStr"/>
+      <c r="T61" s="9" t="inlineStr"/>
+      <c r="U61" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V61" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W61" s="9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="X61" s="9" t="inlineStr">
+        <is>
+          <t>회사, 동료</t>
+        </is>
+      </c>
+      <c r="Y61" s="9" t="inlineStr">
+        <is>
+          <t>같이 빵을 나눠 먹는 동료에서 유래. companion(동료)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-08
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y62"/>
+  <dimension ref="A1:Y63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7788,6 +7788,123 @@
         </is>
       </c>
     </row>
+    <row r="63" ht="60" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H63" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I63" s="9" t="inlineStr">
+        <is>
+          <t>nurture</t>
+        </is>
+      </c>
+      <c r="J63" s="9" t="inlineStr">
+        <is>
+          <t>So my manager really helped nurture my confidence at work. She gave me challenging projects and believed in me, you know? That kind of support makes a huge difference. Now I'm actually thinking about pursuing my own business idea that I've been holding onto for years.</t>
+        </is>
+      </c>
+      <c r="K63" s="9" t="inlineStr">
+        <is>
+          <t>nurture — (성장·발전을) 도와주다, 기르다; pursue — 추구하다, 진행하다</t>
+        </is>
+      </c>
+      <c r="L63" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M63" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N63" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O63" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P63" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q63" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R63" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S63" s="9" t="inlineStr"/>
+      <c r="T63" s="9" t="inlineStr"/>
+      <c r="U63" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V63" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W63" s="9" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="X63" s="9" t="inlineStr">
+        <is>
+          <t>마감 기한</t>
+        </is>
+      </c>
+      <c r="Y63" s="9" t="inlineStr">
+        <is>
+          <t>남북전쟁 포로수용소에서 그 선을 넘으면 사살한다는 경계선에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-09
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y63"/>
+  <dimension ref="A1:Y64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7905,6 +7905,123 @@
         </is>
       </c>
     </row>
+    <row r="64" ht="60" customHeight="1">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H64" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J64" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic story about a young woman named Bathsheba who inherits a farm. She has to manage her business independently, dealing with three different men who want to marry her. It's a fascinating tale about love, responsibility, and making tough decisions.</t>
+        </is>
+      </c>
+      <c r="K64" s="9" t="inlineStr">
+        <is>
+          <t>inherit — 물려받다; manage — 관리하다</t>
+        </is>
+      </c>
+      <c r="L64" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N64" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O64" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P64" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q64" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R64" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S64" s="9" t="inlineStr"/>
+      <c r="T64" s="9" t="inlineStr"/>
+      <c r="U64" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V64" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W64" s="9" t="inlineStr">
+        <is>
+          <t>bankrupt</t>
+        </is>
+      </c>
+      <c r="X64" s="9" t="inlineStr">
+        <is>
+          <t>파산한</t>
+        </is>
+      </c>
+      <c r="Y64" s="9" t="inlineStr">
+        <is>
+          <t>중세 환전상이 파산하면 거래 탁자(banca)를 부수는 관습에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-10
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y64"/>
+  <dimension ref="A1:Y65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8022,6 +8022,123 @@
         </is>
       </c>
     </row>
+    <row r="65" ht="60" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H65" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I65" s="9" t="inlineStr">
+        <is>
+          <t>pedagogical</t>
+        </is>
+      </c>
+      <c r="J65" s="9" t="inlineStr">
+        <is>
+          <t>So our university is redesigning all the classrooms this year, and honestly, it's a great opportunity to think about our teaching methods. The administration wants us to submit proposals showing how we'll use the new spaces, you know? It's not just about picking a room—it's about putting our pedagogical values into practice. I think this change could really transform how we engage with students.</t>
+        </is>
+      </c>
+      <c r="K65" s="9" t="inlineStr">
+        <is>
+          <t>pedagogical — 교육적인, 교수법과 관련된; submit — 제출하다</t>
+        </is>
+      </c>
+      <c r="L65" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M65" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N65" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O65" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P65" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q65" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R65" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S65" s="9" t="inlineStr"/>
+      <c r="T65" s="9" t="inlineStr"/>
+      <c r="U65" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V65" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W65" s="9" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="X65" s="9" t="inlineStr">
+        <is>
+          <t>퀴즈, 시험</t>
+        </is>
+      </c>
+      <c r="Y65" s="9" t="inlineStr">
+        <is>
+          <t>더블린 극장주 Daly가 무의미한 단어를 낙서하면 하루 만에 유행어로 만든 일화에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-11
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y65"/>
+  <dimension ref="A1:Y66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8139,6 +8139,123 @@
         </is>
       </c>
     </row>
+    <row r="66" ht="60" customHeight="1">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H66" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>baptism of fire</t>
+        </is>
+      </c>
+      <c r="J66" s="9" t="inlineStr">
+        <is>
+          <t>So my first week at the new job was pretty intense—I'd say it was a real baptism of fire. They threw me into a major project right away with our biggest client, and honestly, I had no prior experience. But you know what? It actually helped me learn super fast. Sometimes a challenging start is exactly what you need to grow.</t>
+        </is>
+      </c>
+      <c r="K66" s="9" t="inlineStr">
+        <is>
+          <t>baptism of fire — 시련의 첫 경험, 힘든 첫 시작; prior experience — 이전 경험</t>
+        </is>
+      </c>
+      <c r="L66" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M66" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N66" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O66" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P66" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q66" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R66" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S66" s="9" t="inlineStr"/>
+      <c r="T66" s="9" t="inlineStr"/>
+      <c r="U66" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V66" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W66" s="9" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="X66" s="9" t="inlineStr">
+        <is>
+          <t>공황, 극도의 공포</t>
+        </is>
+      </c>
+      <c r="Y66" s="9" t="inlineStr">
+        <is>
+          <t>목신 판(Pan)이 갑자기 나타나 공포를 일으킨다는 신화에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-12
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y66"/>
+  <dimension ref="A1:Y67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8256,6 +8256,123 @@
         </is>
       </c>
     </row>
+    <row r="67" ht="60" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I67" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J67" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic English novel that explores love, ambition, and rural life. The story follows Bathsheba, a young woman who inherits a farm and must manage her responsibilities while dealing with complex relationships. It's a fantastic way to boost your listening skills while enjoying great literature. Why not subscribe to our newsletter and get more resources for learning English?</t>
+        </is>
+      </c>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>inherit — 상속받다; manage — 관리하다, 운영하다</t>
+        </is>
+      </c>
+      <c r="L67" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M67" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N67" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O67" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P67" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q67" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R67" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S67" s="9" t="inlineStr"/>
+      <c r="T67" s="9" t="inlineStr"/>
+      <c r="U67" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V67" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W67" s="9" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="X67" s="9" t="inlineStr">
+        <is>
+          <t>전략</t>
+        </is>
+      </c>
+      <c r="Y67" s="9" t="inlineStr">
+        <is>
+          <t>stratos(군대) + agein(이끌다) → 장군의 기술</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-13
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y67"/>
+  <dimension ref="A1:Y68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8373,6 +8373,123 @@
         </is>
       </c>
     </row>
+    <row r="68" ht="60" customHeight="1">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H68" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J68" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic story that explores themes of love and independence. The narrative follows a strong female character who has to make difficult decisions in her personal life. By listening to this story, you'll not only enjoy great literature but also boost your comprehension skills. So, are you ready to dive into this timeless tale?</t>
+        </is>
+      </c>
+      <c r="K68" s="9" t="inlineStr">
+        <is>
+          <t>narrative — 이야기, 서술; comprehension — 이해, 독해</t>
+        </is>
+      </c>
+      <c r="L68" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M68" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N68" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O68" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P68" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q68" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R68" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S68" s="9" t="inlineStr"/>
+      <c r="T68" s="9" t="inlineStr"/>
+      <c r="U68" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V68" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W68" s="9" t="inlineStr">
+        <is>
+          <t>focus</t>
+        </is>
+      </c>
+      <c r="X68" s="9" t="inlineStr">
+        <is>
+          <t>초점, 집중</t>
+        </is>
+      </c>
+      <c r="Y68" s="9" t="inlineStr">
+        <is>
+          <t>로마 가정의 화덕이 집의 중심이었던 데서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-14
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y68"/>
+  <dimension ref="A1:Y69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8490,6 +8490,123 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="60" customHeight="1">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I69" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J69" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic story about a young woman named Bathsheba who has to manage her farm all by herself. She faces lots of challenges and meets different men along the way. It's a great story to boost your listening and reading skills. Why don't you give it a try?</t>
+        </is>
+      </c>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>manage — 관리하다, 책임지다; boost — 향상시키다, 증진하다</t>
+        </is>
+      </c>
+      <c r="L69" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M69" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N69" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O69" s="9" t="inlineStr">
+        <is>
+          <t>문장 강세와 리듬</t>
+        </is>
+      </c>
+      <c r="P69" s="9" t="inlineStr">
+        <is>
+          <t>내용어(명사·동사·형용사)는 강하게, 기능어(관사·전치사)는 약하게</t>
+        </is>
+      </c>
+      <c r="Q69" s="9" t="inlineStr">
+        <is>
+          <t>I WANT to GO to the STORE | She's WORKING on a NEW project</t>
+        </is>
+      </c>
+      <c r="R69" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S69" s="9" t="inlineStr"/>
+      <c r="T69" s="9" t="inlineStr"/>
+      <c r="U69" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V69" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W69" s="9" t="inlineStr">
+        <is>
+          <t>invest</t>
+        </is>
+      </c>
+      <c r="X69" s="9" t="inlineStr">
+        <is>
+          <t>투자하다</t>
+        </is>
+      </c>
+      <c r="Y69" s="9" t="inlineStr">
+        <is>
+          <t>중세에 왕이 신하에게 땅을 수여할 때 옷(vestis)을 입혀 권한 부여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-15
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y69"/>
+  <dimension ref="A1:Y70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8607,6 +8607,123 @@
         </is>
       </c>
     </row>
+    <row r="70" ht="60" customHeight="1">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H70" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>circumscribe</t>
+        </is>
+      </c>
+      <c r="J70" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you hear about Sarah's new job? She's really excited, but her boss has circumscribed her responsibilities quite a bit. She can only make decisions on small projects. I think she needs to push back and negotiate for more authority if she wants to grow in this role.</t>
+        </is>
+      </c>
+      <c r="K70" s="9" t="inlineStr">
+        <is>
+          <t>circumscribe — 제한하다, 범위를 정하다; push back — 반발하다, 저항하다</t>
+        </is>
+      </c>
+      <c r="L70" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M70" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N70" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O70" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P70" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q70" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R70" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S70" s="9" t="inlineStr"/>
+      <c r="T70" s="9" t="inlineStr"/>
+      <c r="U70" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V70" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W70" s="9" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="X70" s="9" t="inlineStr">
+        <is>
+          <t>위험, 위험을 감수하다</t>
+        </is>
+      </c>
+      <c r="Y70" s="9" t="inlineStr">
+        <is>
+          <t>항해 중 암초 근처를 항행하는 위험에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-16
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y70"/>
+  <dimension ref="A1:Y71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8724,6 +8724,123 @@
         </is>
       </c>
     </row>
+    <row r="71" ht="60" customHeight="1">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="inlineStr">
+        <is>
+          <t>zeugma</t>
+        </is>
+      </c>
+      <c r="J71" s="9" t="inlineStr">
+        <is>
+          <t>So, have you ever heard of zeugma? It's actually a really cool wordplay technique where one word has different meanings in each phrase. For example, you might say someone 'lost their keys and their temper'—same word, totally different situations. It's a clever way to add humor to your writing or presentations at work.</t>
+        </is>
+      </c>
+      <c r="K71" s="9" t="inlineStr">
+        <is>
+          <t>zeugma — 하나의 단어가 다양한 의미로 쓰이는 말장난; technique — 기법, 기술</t>
+        </is>
+      </c>
+      <c r="L71" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M71" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N71" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O71" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P71" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q71" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R71" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S71" s="9" t="inlineStr"/>
+      <c r="T71" s="9" t="inlineStr"/>
+      <c r="U71" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V71" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W71" s="9" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="X71" s="9" t="inlineStr">
+        <is>
+          <t>예산</t>
+        </is>
+      </c>
+      <c r="Y71" s="9" t="inlineStr">
+        <is>
+          <t>재무장관이 예산서를 담은 가죽 가방(bougette)을 들고 의회에 출석한 데서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-17
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y71"/>
+  <dimension ref="A1:Y72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8841,6 +8841,123 @@
         </is>
       </c>
     </row>
+    <row r="72" ht="60" customHeight="1">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="inlineStr">
+        <is>
+          <t>lackadaisical</t>
+        </is>
+      </c>
+      <c r="J72" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you notice how the team's performance was really lackadaisical during that game? I mean, they just weren't motivated at all. The coach was frustrated because even the best players seemed lazy and unfocused. I guess everyone has those days when they lack enthusiasm, right?</t>
+        </is>
+      </c>
+      <c r="K72" s="9" t="inlineStr">
+        <is>
+          <t>lackadaisical — 무기력한, 열정 없는; motivated — 동기 부여된, 동기가 있는</t>
+        </is>
+      </c>
+      <c r="L72" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M72" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N72" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O72" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P72" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q72" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R72" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S72" s="9" t="inlineStr"/>
+      <c r="T72" s="9" t="inlineStr"/>
+      <c r="U72" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V72" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W72" s="9" t="inlineStr">
+        <is>
+          <t>magazine</t>
+        </is>
+      </c>
+      <c r="X72" s="9" t="inlineStr">
+        <is>
+          <t>잡지, 탄창</t>
+        </is>
+      </c>
+      <c r="Y72" s="9" t="inlineStr">
+        <is>
+          <t>지식·정보를 저장해 두는 '창고'라는 의미로 출판물에 사용됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-18
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y72"/>
+  <dimension ref="A1:Y73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8958,6 +8958,123 @@
         </is>
       </c>
     </row>
+    <row r="73" ht="60" customHeight="1">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="inlineStr">
+        <is>
+          <t>oxymoron</t>
+        </is>
+      </c>
+      <c r="J73" s="9" t="inlineStr">
+        <is>
+          <t>You know, I think our new marketing campaign is kind of an oxymoron. We're trying to sell expensive eco-friendly products, but most people can't afford them, right? It's like we're promoting sustainability while making it exclusive. Anyway, the team says this strategy will resonate with wealthy consumers, so let's see how it goes.</t>
+        </is>
+      </c>
+      <c r="K73" s="9" t="inlineStr">
+        <is>
+          <t>oxymoron — 모순적인 표현; resonate — (대상에게) 호감을 얻다, 반향을 일으키다</t>
+        </is>
+      </c>
+      <c r="L73" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M73" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N73" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O73" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P73" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q73" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R73" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S73" s="9" t="inlineStr"/>
+      <c r="T73" s="9" t="inlineStr"/>
+      <c r="U73" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V73" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W73" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X73" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y73" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-19
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y73"/>
+  <dimension ref="A1:Y74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9075,6 +9075,123 @@
         </is>
       </c>
     </row>
+    <row r="74" ht="60" customHeight="1">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>현재완료 vs 단순과거</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Present Perfect vs Simple Past</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>balmy</t>
+        </is>
+      </c>
+      <c r="J74" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you see the weather forecast for this weekend? It's supposed to be really balmy—you know, warm and pleasant. Perfect weather for that outdoor concert we've been planning. We should definitely bring some snacks and chairs to enjoy the evening.</t>
+        </is>
+      </c>
+      <c r="K74" s="9" t="inlineStr">
+        <is>
+          <t>balmy — 따뜻하고 쾌적한; forecast — 날씨 예보</t>
+        </is>
+      </c>
+      <c r="L74" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M74" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N74" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O74" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P74" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q74" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R74" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S74" s="9" t="inlineStr"/>
+      <c r="T74" s="9" t="inlineStr"/>
+      <c r="U74" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V74" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W74" s="9" t="inlineStr">
+        <is>
+          <t>serendipity</t>
+        </is>
+      </c>
+      <c r="X74" s="9" t="inlineStr">
+        <is>
+          <t>뜻밖의 행운</t>
+        </is>
+      </c>
+      <c r="Y74" s="9" t="inlineStr">
+        <is>
+          <t>세 왕자가 우연히 훌륭한 발견을 하는 동화에서 Horace Walpole이 만든 단어</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-20
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y74"/>
+  <dimension ref="A1:Y75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9192,6 +9192,123 @@
         </is>
       </c>
     </row>
+    <row r="75" ht="60" customHeight="1">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>능력·공손 조동사</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: can / could — 능력과 공손</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>divulge</t>
+        </is>
+      </c>
+      <c r="J75" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you hear about the new product launch? The CEO promised not to divulge any details before the official announcement next month. But honestly, I think some employees have already leaked information online. Management is pretty upset about it.</t>
+        </is>
+      </c>
+      <c r="K75" s="9" t="inlineStr">
+        <is>
+          <t>divulge — (비밀 정보를) 공개하다, 드러내다; leak — 새어나가게 하다, 유출하다</t>
+        </is>
+      </c>
+      <c r="L75" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M75" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N75" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O75" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P75" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q75" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R75" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S75" s="9" t="inlineStr"/>
+      <c r="T75" s="9" t="inlineStr"/>
+      <c r="U75" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V75" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W75" s="9" t="inlineStr">
+        <is>
+          <t>berserk</t>
+        </is>
+      </c>
+      <c r="X75" s="9" t="inlineStr">
+        <is>
+          <t>극도로 흥분한, 폭주하는</t>
+        </is>
+      </c>
+      <c r="Y75" s="9" t="inlineStr">
+        <is>
+          <t>전투에서 곰 가죽을 입고 광분하던 바이킹 전사에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-21
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y75"/>
+  <dimension ref="A1:Y76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9309,6 +9309,123 @@
         </is>
       </c>
     </row>
+    <row r="76" ht="60" customHeight="1">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>실현 가능한 조건문</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>First Conditional</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H76" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I76" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J76" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at 'Far From the Madding Crowd,' a classic story that explores love and relationships in rural England. The main character, Bathsheba, has to manage her farm while dealing with three very different men who want to marry her. It's a fascinating tale about independence and the challenges of making difficult choices in life.</t>
+        </is>
+      </c>
+      <c r="K76" s="9" t="inlineStr">
+        <is>
+          <t>manage — 관리하다; independence — 독립, 자주성</t>
+        </is>
+      </c>
+      <c r="L76" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M76" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N76" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O76" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P76" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q76" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R76" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S76" s="9" t="inlineStr"/>
+      <c r="T76" s="9" t="inlineStr"/>
+      <c r="U76" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V76" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W76" s="9" t="inlineStr">
+        <is>
+          <t>boycott</t>
+        </is>
+      </c>
+      <c r="X76" s="9" t="inlineStr">
+        <is>
+          <t>불매운동, 거부하다</t>
+        </is>
+      </c>
+      <c r="Y76" s="9" t="inlineStr">
+        <is>
+          <t>1880년 소작인들이 Boycott을 집단 거부한 사건에서 단어화</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-22
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y76"/>
+  <dimension ref="A1:Y77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9426,6 +9426,123 @@
         </is>
       </c>
     </row>
+    <row r="77" ht="60" customHeight="1">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>수동태</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Passive Voice</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H77" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I77" s="9" t="inlineStr">
+        <is>
+          <t>august</t>
+        </is>
+      </c>
+      <c r="J77" s="9" t="inlineStr">
+        <is>
+          <t>So, the word 'august' means something really grand and impressive, you know? Like, when you walk into an old palace with those high ceilings and fancy decorations, that's an august setting. It actually comes from the Roman calendar—they named the month of August after Emperor Augustus. Pretty cool, right?</t>
+        </is>
+      </c>
+      <c r="K77" s="9" t="inlineStr">
+        <is>
+          <t>august — 웅장한, 위엄 있는; palace — 궁전</t>
+        </is>
+      </c>
+      <c r="L77" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M77" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N77" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O77" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P77" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q77" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R77" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S77" s="9" t="inlineStr"/>
+      <c r="T77" s="9" t="inlineStr"/>
+      <c r="U77" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V77" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W77" s="9" t="inlineStr">
+        <is>
+          <t>mentor</t>
+        </is>
+      </c>
+      <c r="X77" s="9" t="inlineStr">
+        <is>
+          <t>멘토, 스승</t>
+        </is>
+      </c>
+      <c r="Y77" s="9" t="inlineStr">
+        <is>
+          <t>오디세우스가 트로이 전쟁 중 아들 텔레마코스 교육을 맡긴 현자의 이름에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-23
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y77"/>
+  <dimension ref="A1:Y78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9543,6 +9543,123 @@
         </is>
       </c>
     </row>
+    <row r="78" ht="60" customHeight="1">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>관사</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Articles: a / an / the</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="inlineStr">
+        <is>
+          <t>prowess</t>
+        </is>
+      </c>
+      <c r="J78" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you see Sarah's presentation at the meeting? Her speaking prowess really impressed everyone, including the boss. I mean, she explained that complicated project so clearly. You know, it's not just about having talent—you gotta practice and develop your skills over time.</t>
+        </is>
+      </c>
+      <c r="K78" s="9" t="inlineStr">
+        <is>
+          <t>prowess — 뛰어난 능력/기술; develop — 발전시키다/개발하다</t>
+        </is>
+      </c>
+      <c r="L78" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N78" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O78" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P78" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q78" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R78" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S78" s="9" t="inlineStr"/>
+      <c r="T78" s="9" t="inlineStr"/>
+      <c r="U78" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V78" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W78" s="9" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="X78" s="9" t="inlineStr">
+        <is>
+          <t>경쟁자</t>
+        </is>
+      </c>
+      <c r="Y78" s="9" t="inlineStr">
+        <is>
+          <t>같은 강(rivus) 물을 사용하는 이웃 사이의 경쟁 관계에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-24
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y78"/>
+  <dimension ref="A1:Y79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9660,6 +9660,123 @@
         </is>
       </c>
     </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>강조 도치</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>Inversion for Emphasis</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I79" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J79" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic story called 'Far From the Madding Crowd'. It's a brilliant novel that explores themes of love and ambition in rural England. As you listen to this story, you'll boost your comprehension skills while enjoying some wonderful English literature. Make sure to follow along and pick up new vocabulary!</t>
+        </is>
+      </c>
+      <c r="K79" s="9" t="inlineStr">
+        <is>
+          <t>comprehension — 이해력, 이해; ambition — 야망, 포부</t>
+        </is>
+      </c>
+      <c r="L79" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M79" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N79" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O79" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P79" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q79" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R79" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S79" s="9" t="inlineStr"/>
+      <c r="T79" s="9" t="inlineStr"/>
+      <c r="U79" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V79" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W79" s="9" t="inlineStr">
+        <is>
+          <t>travel</t>
+        </is>
+      </c>
+      <c r="X79" s="9" t="inlineStr">
+        <is>
+          <t>여행하다</t>
+        </is>
+      </c>
+      <c r="Y79" s="9" t="inlineStr">
+        <is>
+          <t>중세 여행이 고문(tripalium)처럼 고달팠던 데서 travail(고통)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-25
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y79"/>
+  <dimension ref="A1:Y80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9777,6 +9777,123 @@
         </is>
       </c>
     </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>과거완료</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Past Perfect Tense</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J80" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic story that explores themes of love and ambition in rural England. The main character, Bathsheba, is an independent woman who manages her own farm, which was quite unusual back then. As you listen to this story, you'll pick up lots of useful vocabulary about farming and relationships. So sit back, relax, and enjoy this timeless tale!</t>
+        </is>
+      </c>
+      <c r="K80" s="9" t="inlineStr">
+        <is>
+          <t>independent — 독립적인; manages — 관리하다</t>
+        </is>
+      </c>
+      <c r="L80" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N80" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O80" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P80" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q80" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R80" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S80" s="9" t="inlineStr"/>
+      <c r="T80" s="9" t="inlineStr"/>
+      <c r="U80" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V80" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W80" s="9" t="inlineStr">
+        <is>
+          <t>enthusiasm</t>
+        </is>
+      </c>
+      <c r="X80" s="9" t="inlineStr">
+        <is>
+          <t>열정, 열의</t>
+        </is>
+      </c>
+      <c r="Y80" s="9" t="inlineStr">
+        <is>
+          <t>en(안에) + theos(신) → 신에게 감화받은 열정 상태</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-26
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y80"/>
+  <dimension ref="A1:Y81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9894,6 +9894,123 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>의무·충고 조동사</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: should / ought to / had better</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I81" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J81" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at Far From the Madding Crowd, a classic novel that explores love and relationships in rural England. The story follows Bathsheba, a strong-willed woman who manages her own farm and has to navigate complicated feelings for three different men. It's a brilliant tale about independence and the challenges people face when they pursue their own ambitions.</t>
+        </is>
+      </c>
+      <c r="K81" s="9" t="inlineStr">
+        <is>
+          <t>navigate — (상황을) 헤쳐나가다, 대처하다; ambitious — 야심 있는, 포부가 있는</t>
+        </is>
+      </c>
+      <c r="L81" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N81" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O81" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P81" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q81" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R81" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S81" s="9" t="inlineStr"/>
+      <c r="T81" s="9" t="inlineStr"/>
+      <c r="U81" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V81" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W81" s="9" t="inlineStr">
+        <is>
+          <t>lucid</t>
+        </is>
+      </c>
+      <c r="X81" s="9" t="inlineStr">
+        <is>
+          <t>명확한, 이해하기 쉬운</t>
+        </is>
+      </c>
+      <c r="Y81" s="9" t="inlineStr">
+        <is>
+          <t>lux(빛)과 동근 → 명확하고 투명한 사고</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-28
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y81"/>
+  <dimension ref="A1:Y82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10011,6 +10011,123 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="60" customHeight="1">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>Second Conditional</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Far From the Madding Crowd</t>
+        </is>
+      </c>
+      <c r="J82" s="9" t="inlineStr">
+        <is>
+          <t>Far From the Madding Crowd is a classic story that follows Bathsheba Everdene, a strong and independent woman living in the English countryside. Throughout the narrative, she faces several challenges that test her character and relationships. This BBC Learning English programme helps you boost your listening skills while enjoying great literature. Why not sign up to our newsletter for more learning resources?</t>
+        </is>
+      </c>
+      <c r="K82" s="9" t="inlineStr">
+        <is>
+          <t>independent — 독립적인; narrative — 이야기, 서술</t>
+        </is>
+      </c>
+      <c r="L82" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N82" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P82" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q82" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R82" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S82" s="9" t="inlineStr"/>
+      <c r="T82" s="9" t="inlineStr"/>
+      <c r="U82" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V82" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W82" s="9" t="inlineStr">
+        <is>
+          <t>colleague</t>
+        </is>
+      </c>
+      <c r="X82" s="9" t="inlineStr">
+        <is>
+          <t>동료</t>
+        </is>
+      </c>
+      <c r="Y82" s="9" t="inlineStr">
+        <is>
+          <t>col(함께) + legare(선택하다/보내다) → 같이 선발된 동료</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-29
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y82"/>
+  <dimension ref="A1:Y83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10128,6 +10128,123 @@
         </is>
       </c>
     </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>간접화법</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>Reported Speech</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I83" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Murders in the Rue Morgue</t>
+        </is>
+      </c>
+      <c r="J83" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic mystery story called 'The Murders in the Rue Morgue.' You'll learn nine different ways to use the word 'run' while enjoying this exciting tale. It's a perfect way to improve your English vocabulary in just five minutes. Plus, we have lots of other podcasts available to help you keep learning!</t>
+        </is>
+      </c>
+      <c r="K83" s="9" t="inlineStr">
+        <is>
+          <t>mystery — 미스터리, 수수께끼; podcast — 팟캐스트, 음성 방송</t>
+        </is>
+      </c>
+      <c r="L83" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N83" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O83" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P83" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q83" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R83" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S83" s="9" t="inlineStr"/>
+      <c r="T83" s="9" t="inlineStr"/>
+      <c r="U83" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V83" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W83" s="9" t="inlineStr">
+        <is>
+          <t>quarantine</t>
+        </is>
+      </c>
+      <c r="X83" s="9" t="inlineStr">
+        <is>
+          <t>격리, 검역</t>
+        </is>
+      </c>
+      <c r="Y83" s="9" t="inlineStr">
+        <is>
+          <t>14세기 흑사병 때 선박을 40일간 격리한 베네치아 방역 정책에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-30
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y84"/>
+  <dimension ref="A1:Y85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10362,6 +10362,123 @@
         </is>
       </c>
     </row>
+    <row r="85" ht="60" customHeight="1">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>가정법 현재 (요구·제안 구문)</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Subjunctive Mood</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I85" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Murders in the Rue Morgue</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic mystery story and discover how the word 'run' is used in different ways. The story involves a detective who has to run through clues to solve a brutal crime. You'll pick up practical language while enjoying this thrilling tale, so stick around!</t>
+        </is>
+      </c>
+      <c r="K85" s="9" t="inlineStr">
+        <is>
+          <t>run through — ~을 빠르게 검토하다; brutal — 잔인한</t>
+        </is>
+      </c>
+      <c r="L85" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N85" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O85" s="9" t="inlineStr">
+        <is>
+          <t>억양: 의문문</t>
+        </is>
+      </c>
+      <c r="P85" s="9" t="inlineStr">
+        <is>
+          <t>Yes/No 질문은 끝이 올라가고 ↗, Wh- 질문은 끝이 내려감 ↘</t>
+        </is>
+      </c>
+      <c r="Q85" s="9" t="inlineStr">
+        <is>
+          <t>Are you READY? ↗ | Where are you GOING? ↘ | Did you SEE it? ↗</t>
+        </is>
+      </c>
+      <c r="R85" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S85" s="9" t="inlineStr"/>
+      <c r="T85" s="9" t="inlineStr"/>
+      <c r="U85" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V85" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W85" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X85" s="9" t="inlineStr">
+        <is>
+          <t>급여</t>
+        </is>
+      </c>
+      <c r="Y85" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사의 소금 급여에서. '소금값 못하는 사람'이라는 표현도 여기서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-08-31
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y85"/>
+  <dimension ref="A1:Y86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10479,6 +10479,123 @@
         </is>
       </c>
     </row>
+    <row r="86" ht="60" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>미래 표현 3가지</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>Future Tenses: will / going to / present continuous</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G86" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H86" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I86" s="9" t="inlineStr">
+        <is>
+          <t>gumption</t>
+        </is>
+      </c>
+      <c r="J86" s="9" t="inlineStr">
+        <is>
+          <t>You know, it really takes gumption to start your own business these days. My friend Sarah quit her job last year to launch a startup—I mean, that's a bold move! She had the courage and confidence to take that risk, and honestly, that kind of determination is pretty inspiring. I think more people need that gumption to pursue their dreams.</t>
+        </is>
+      </c>
+      <c r="K86" s="9" t="inlineStr">
+        <is>
+          <t>gumption — 용기와 자신감; bold move — 대담한 결정</t>
+        </is>
+      </c>
+      <c r="L86" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M86" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N86" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>r vs l 구분</t>
+        </is>
+      </c>
+      <c r="P86" s="9" t="inlineStr">
+        <is>
+          <t>r은 혀를 말아 입천장에 닿지 않게, l은 혀끝을 윗잇몸에 확실히 댐</t>
+        </is>
+      </c>
+      <c r="Q86" s="9" t="inlineStr">
+        <is>
+          <t>really /ríːli/ | rally /réli/ | river /rívər/ | liver /lívər/</t>
+        </is>
+      </c>
+      <c r="R86" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S86" s="9" t="inlineStr"/>
+      <c r="T86" s="9" t="inlineStr"/>
+      <c r="U86" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V86" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W86" s="9" t="inlineStr">
+        <is>
+          <t>sincere</t>
+        </is>
+      </c>
+      <c r="X86" s="9" t="inlineStr">
+        <is>
+          <t>진실한, 진심 어린</t>
+        </is>
+      </c>
+      <c r="Y86" s="9" t="inlineStr">
+        <is>
+          <t>로마 조각가가 결함을 밀랍으로 숨겼는데, 최고 작품은 밀랍 없이(sine cera) 완성됨</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-01
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y86"/>
+  <dimension ref="A1:Y87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10596,6 +10596,123 @@
         </is>
       </c>
     </row>
+    <row r="87" ht="60" customHeight="1">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>의무·필요 조동사</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>Modal Verbs: must / have to / need to</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Murders in the Rue Morgue</t>
+        </is>
+      </c>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>Today we're going to explore a classic mystery story and learn different ways to use the word 'run'. You'll pick up nine useful expressions in just five minutes. It's a great way to expand your vocabulary while enjoying an entertaining tale. Don't forget to check out our other podcasts for more learning resources!</t>
+        </is>
+      </c>
+      <c r="K87" s="9" t="inlineStr">
+        <is>
+          <t>expand — 확대하다, 늘리다; entertaining — 재미있는, 흥미로운</t>
+        </is>
+      </c>
+      <c r="L87" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M87" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N87" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O87" s="9" t="inlineStr">
+        <is>
+          <t>f vs p 구분</t>
+        </is>
+      </c>
+      <c r="P87" s="9" t="inlineStr">
+        <is>
+          <t>f는 윗니를 아랫입술에 대고 바람, p는 두 입술로 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q87" s="9" t="inlineStr">
+        <is>
+          <t>food /fuːd/ | pool /puːl/ | fee /fiː/ | pea /piː/</t>
+        </is>
+      </c>
+      <c r="R87" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S87" s="9" t="inlineStr"/>
+      <c r="T87" s="9" t="inlineStr"/>
+      <c r="U87" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V87" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W87" s="9" t="inlineStr">
+        <is>
+          <t>salary</t>
+        </is>
+      </c>
+      <c r="X87" s="9" t="inlineStr">
+        <is>
+          <t>급여, 봉급</t>
+        </is>
+      </c>
+      <c r="Y87" s="9" t="inlineStr">
+        <is>
+          <t>로마 병사는 소금(sal)으로 급여를 받았음. salt와 같은 어근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-02
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y87"/>
+  <dimension ref="A1:Y88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10713,6 +10713,123 @@
         </is>
       </c>
     </row>
+    <row r="88" ht="60" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>가정법 과거완료·혼합</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>Third Conditional &amp; Mixed Conditionals</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G88" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H88" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I88" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: The Murders in the Rue Morgue</t>
+        </is>
+      </c>
+      <c r="J88" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic mystery story, 'The Murders in the Rue Morgue,' and exploring different uses of the word 'run.' You'll learn how this common verb appears throughout the story—like when a character runs away or when an investigation runs into problems. By the end, you'll understand nine different meanings and can run through examples yourself.</t>
+        </is>
+      </c>
+      <c r="K88" s="9" t="inlineStr">
+        <is>
+          <t>investigation — 조사, 수사; classic — 고전의, 고전 작품</t>
+        </is>
+      </c>
+      <c r="L88" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M88" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N88" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O88" s="9" t="inlineStr">
+        <is>
+          <t>v vs b 구분</t>
+        </is>
+      </c>
+      <c r="P88" s="9" t="inlineStr">
+        <is>
+          <t>v는 윗니를 아랫입술에 대고 진동, b는 두 입술로 막아 터뜨림</t>
+        </is>
+      </c>
+      <c r="Q88" s="9" t="inlineStr">
+        <is>
+          <t>very /véri/ | berry /béri/ | vest /vest/ | best /best/</t>
+        </is>
+      </c>
+      <c r="R88" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S88" s="9" t="inlineStr"/>
+      <c r="T88" s="9" t="inlineStr"/>
+      <c r="U88" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V88" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W88" s="9" t="inlineStr">
+        <is>
+          <t>muscle</t>
+        </is>
+      </c>
+      <c r="X88" s="9" t="inlineStr">
+        <is>
+          <t>근육</t>
+        </is>
+      </c>
+      <c r="Y88" s="9" t="inlineStr">
+        <is>
+          <t>팔을 구부릴 때 근육이 움직이는 모습이 쥐처럼 보인다 하여</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-03
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y88"/>
+  <dimension ref="A1:Y89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10830,6 +10830,123 @@
         </is>
       </c>
     </row>
+    <row r="89" ht="60" customHeight="1">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B89" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>관계절</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Relative Clauses: defining vs non-defining</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H89" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I89" s="9" t="inlineStr">
+        <is>
+          <t>recalcitrant</t>
+        </is>
+      </c>
+      <c r="J89" s="9" t="inlineStr">
+        <is>
+          <t>My boss gave me a recalcitrant printer to fix, and honestly, it's been a nightmare. The thing refuses to cooperate no matter what I do. I'm thinking about just replacing it because some equipment is just too stubborn to work with.</t>
+        </is>
+      </c>
+      <c r="K89" s="9" t="inlineStr">
+        <is>
+          <t>recalcitrant — 고집 센, 말을 안 듣는; cooperate — 협력하다, 협조하다</t>
+        </is>
+      </c>
+      <c r="L89" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M89" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N89" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O89" s="9" t="inlineStr">
+        <is>
+          <t>th 유성음 /ð/</t>
+        </is>
+      </c>
+      <c r="P89" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 목소리 진동</t>
+        </is>
+      </c>
+      <c r="Q89" s="9" t="inlineStr">
+        <is>
+          <t>the /ðə/ | this /ðɪs/ | that /ðæt/ | mother /mʌðər/</t>
+        </is>
+      </c>
+      <c r="R89" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S89" s="9" t="inlineStr"/>
+      <c r="T89" s="9" t="inlineStr"/>
+      <c r="U89" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V89" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W89" s="9" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="X89" s="9" t="inlineStr">
+        <is>
+          <t>후보자</t>
+        </is>
+      </c>
+      <c r="Y89" s="9" t="inlineStr">
+        <is>
+          <t>로마 선거 출마자는 순결을 상징하는 흰 토가(candida)를 입었음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-04
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y89"/>
+  <dimension ref="A1:Y90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10947,6 +10947,123 @@
         </is>
       </c>
     </row>
+    <row r="90" ht="60" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B90" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>시간 전치사</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Time: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G90" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H90" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I90" s="9" t="inlineStr">
+        <is>
+          <t>apiary</t>
+        </is>
+      </c>
+      <c r="J90" s="9" t="inlineStr">
+        <is>
+          <t>So my sister-in-law actually runs a small apiary in our backyard. She keeps about twenty colonies of bees there and sells the honey at the local farmers market. It's pretty cool because we always have fresh honey at home, and she says it's a really therapeutic hobby too.</t>
+        </is>
+      </c>
+      <c r="K90" s="9" t="inlineStr">
+        <is>
+          <t>apiary — 양봉장; colony — 집단, 식민지</t>
+        </is>
+      </c>
+      <c r="L90" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M90" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N90" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O90" s="9" t="inlineStr">
+        <is>
+          <t>th 무성음 /θ/</t>
+        </is>
+      </c>
+      <c r="P90" s="9" t="inlineStr">
+        <is>
+          <t>혀끝을 윗니 사이에 살짝 내밀고 바람만 내보냄</t>
+        </is>
+      </c>
+      <c r="Q90" s="9" t="inlineStr">
+        <is>
+          <t>think /θɪŋk/ | three /θriː/ | health /helθ/ | month /mʌnθ/</t>
+        </is>
+      </c>
+      <c r="R90" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S90" s="9" t="inlineStr"/>
+      <c r="T90" s="9" t="inlineStr"/>
+      <c r="U90" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V90" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W90" s="9" t="inlineStr">
+        <is>
+          <t>disaster</t>
+        </is>
+      </c>
+      <c r="X90" s="9" t="inlineStr">
+        <is>
+          <t>재앙, 참사</t>
+        </is>
+      </c>
+      <c r="Y90" s="9" t="inlineStr">
+        <is>
+          <t>별의 위치가 나쁘면 재앙이 온다는 점성술 믿음에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-05
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y90"/>
+  <dimension ref="A1:Y91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11064,6 +11064,123 @@
         </is>
       </c>
     </row>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>생략과 대용</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Ellipsis and Substitution</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H91" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I91" s="9" t="inlineStr">
+        <is>
+          <t>matriculate</t>
+        </is>
+      </c>
+      <c r="J91" s="9" t="inlineStr">
+        <is>
+          <t>Hey, did you hear that Sarah finally matriculated at Harvard? Yeah, she enrolled last month and starts classes next week. A lot of students take a gap year before matriculating, but she was eager to jump right in. It's a big milestone for her family.</t>
+        </is>
+      </c>
+      <c r="K91" s="9" t="inlineStr">
+        <is>
+          <t>matriculate — (대학에) 입학하다, 등록하다; gap year — 휴학년, 진학 전 쉬는 기간</t>
+        </is>
+      </c>
+      <c r="L91" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M91" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N91" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O91" s="9" t="inlineStr">
+        <is>
+          <t>짧은 모음 vs 긴 모음</t>
+        </is>
+      </c>
+      <c r="P91" s="9" t="inlineStr">
+        <is>
+          <t>ship /ɪ/ vs sheep /iː/ — 입 모양과 길이 모두 다름</t>
+        </is>
+      </c>
+      <c r="Q91" s="9" t="inlineStr">
+        <is>
+          <t>ship /ʃɪp/ | sheep /ʃiːp/ | hit /hɪt/ | heat /hiːt/</t>
+        </is>
+      </c>
+      <c r="R91" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S91" s="9" t="inlineStr"/>
+      <c r="T91" s="9" t="inlineStr"/>
+      <c r="U91" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V91" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W91" s="9" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="X91" s="9" t="inlineStr">
+        <is>
+          <t>회사, 동료</t>
+        </is>
+      </c>
+      <c r="Y91" s="9" t="inlineStr">
+        <is>
+          <t>같이 빵을 나눠 먹는 동료에서 유래. companion(동료)과 동근</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-06
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y91"/>
+  <dimension ref="A1:Y92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11181,6 +11181,123 @@
         </is>
       </c>
     </row>
+    <row r="92" ht="60" customHeight="1">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>단순현재 vs 현재진행</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>Present Simple vs Present Continuous</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G92" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H92" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I92" s="9" t="inlineStr">
+        <is>
+          <t>inexorable</t>
+        </is>
+      </c>
+      <c r="J92" s="9" t="inlineStr">
+        <is>
+          <t>You know, the changing seasons remind us of something really important. Time just keeps moving forward—it's inexorable, you can't stop it or slow it down. That's why ancient people built monuments like Stonehenge to track the seasons. Understanding these cycles helped them plan their work and prepare for what comes next.</t>
+        </is>
+      </c>
+      <c r="K92" s="9" t="inlineStr">
+        <is>
+          <t>inexorable — 막을 수 없는, 피할 수 없는; track — 추적하다, 기록하다</t>
+        </is>
+      </c>
+      <c r="L92" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M92" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N92" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O92" s="9" t="inlineStr">
+        <is>
+          <t>어말 자음 탈락 방지</t>
+        </is>
+      </c>
+      <c r="P92" s="9" t="inlineStr">
+        <is>
+          <t>한국어는 받침 뒤 모음을 붙이는 경향 — 마지막 자음만 닫고 끝내기</t>
+        </is>
+      </c>
+      <c r="Q92" s="9" t="inlineStr">
+        <is>
+          <t>fact /fækt/ | next /nekst/ | helped /helpt/ | asked /æskt/</t>
+        </is>
+      </c>
+      <c r="R92" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S92" s="9" t="inlineStr"/>
+      <c r="T92" s="9" t="inlineStr"/>
+      <c r="U92" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V92" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W92" s="9" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="X92" s="9" t="inlineStr">
+        <is>
+          <t>계산하다</t>
+        </is>
+      </c>
+      <c r="Y92" s="9" t="inlineStr">
+        <is>
+          <t>로마인이 주판 대신 조약돌(calculus)로 계산했음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-07
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y92"/>
+  <dimension ref="A1:Y93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11298,6 +11298,123 @@
         </is>
       </c>
     </row>
+    <row r="93" ht="60" customHeight="1">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B93" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>구동사 (비즈니스)</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>Phrasal Verbs – Business Context</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H93" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I93" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Orpheus and Eurydice</t>
+        </is>
+      </c>
+      <c r="J93" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring a classic Greek myth about Orpheus and Eurydice. This story teaches us about love and loss through beautiful poetry and music. You'll learn thirteen different uses of the word 'long' while enjoying this timeless tale. It's a perfect way to improve your English in just five minutes!</t>
+        </is>
+      </c>
+      <c r="K93" s="9" t="inlineStr">
+        <is>
+          <t>timeless — 시대를 초월한, 영원한; myth — 신화</t>
+        </is>
+      </c>
+      <c r="L93" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M93" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N93" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O93" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 명사</t>
+        </is>
+      </c>
+      <c r="P93" s="9" t="inlineStr">
+        <is>
+          <t>명사는 보통 첫 음절 강세 — REcord, PROtest, PERmit</t>
+        </is>
+      </c>
+      <c r="Q93" s="9" t="inlineStr">
+        <is>
+          <t>REcord | PROtest | PERmit | CONtent</t>
+        </is>
+      </c>
+      <c r="R93" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S93" s="9" t="inlineStr"/>
+      <c r="T93" s="9" t="inlineStr"/>
+      <c r="U93" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V93" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W93" s="9" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="X93" s="9" t="inlineStr">
+        <is>
+          <t>마감 기한</t>
+        </is>
+      </c>
+      <c r="Y93" s="9" t="inlineStr">
+        <is>
+          <t>남북전쟁 포로수용소에서 그 선을 넘으면 사살한다는 경계선에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-08
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y93"/>
+  <dimension ref="A1:Y94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11415,6 +11415,123 @@
         </is>
       </c>
     </row>
+    <row r="94" ht="60" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>비교급·최상급</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
+        <is>
+          <t>Comparative and Superlative Adjectives</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F94" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G94" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H94" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I94" s="9" t="inlineStr">
+        <is>
+          <t>magnanimous</t>
+        </is>
+      </c>
+      <c r="J94" s="9" t="inlineStr">
+        <is>
+          <t>When your coworker made that mistake on the project, you handled it really well. You didn't get angry or blame them. That's being magnanimous—showing kindness even when someone messes up. In business, that kind of attitude actually builds stronger teams and better relationships.</t>
+        </is>
+      </c>
+      <c r="K94" s="9" t="inlineStr">
+        <is>
+          <t>magnanimous — 관대한, 너그러운; coworker — 직장 동료</t>
+        </is>
+      </c>
+      <c r="L94" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M94" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N94" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O94" s="9" t="inlineStr">
+        <is>
+          <t>단어 강세: 2음절 동사</t>
+        </is>
+      </c>
+      <c r="P94" s="9" t="inlineStr">
+        <is>
+          <t>동사는 보통 두 번째 음절 강세 — reCORD, proTEST, perMIT</t>
+        </is>
+      </c>
+      <c r="Q94" s="9" t="inlineStr">
+        <is>
+          <t>reCORD | proTEST | perMIT | conTENT</t>
+        </is>
+      </c>
+      <c r="R94" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S94" s="9" t="inlineStr"/>
+      <c r="T94" s="9" t="inlineStr"/>
+      <c r="U94" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V94" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W94" s="9" t="inlineStr">
+        <is>
+          <t>bankrupt</t>
+        </is>
+      </c>
+      <c r="X94" s="9" t="inlineStr">
+        <is>
+          <t>파산한</t>
+        </is>
+      </c>
+      <c r="Y94" s="9" t="inlineStr">
+        <is>
+          <t>중세 환전상이 파산하면 거래 탁자(banca)를 부수는 관습에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-09
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y94"/>
+  <dimension ref="A1:Y95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11532,6 +11532,123 @@
         </is>
       </c>
     </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B95" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>장소 전치사</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Prepositions of Place: at / in / on / by</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H95" s="9" t="inlineStr">
+        <is>
+          <t>Merriam-Webster Word of the Day</t>
+        </is>
+      </c>
+      <c r="I95" s="9" t="inlineStr">
+        <is>
+          <t>stigma</t>
+        </is>
+      </c>
+      <c r="J95" s="9" t="inlineStr">
+        <is>
+          <t>You know, there's still a lot of stigma around people with mental health issues, even though it's becoming more accepted. Companies are trying to tackle this by creating more supportive work environments. It's really important that we challenge these unfair beliefs because they can seriously impact people's lives and careers.</t>
+        </is>
+      </c>
+      <c r="K95" s="9" t="inlineStr">
+        <is>
+          <t>stigma — 편견, 오명; tackle — 대처하다, 해결하다</t>
+        </is>
+      </c>
+      <c r="L95" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M95" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N95" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O95" s="9" t="inlineStr">
+        <is>
+          <t>-ed 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P95" s="9" t="inlineStr">
+        <is>
+          <t>/t/: 무성음 뒤 | /d/: 유성음 뒤 | /ɪd/: t·d로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q95" s="9" t="inlineStr">
+        <is>
+          <t>worked /wɜːrkt/ | called /kɔːld/ | wanted /wɒntɪd/ | needed /niːdɪd/</t>
+        </is>
+      </c>
+      <c r="R95" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S95" s="9" t="inlineStr"/>
+      <c r="T95" s="9" t="inlineStr"/>
+      <c r="U95" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V95" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W95" s="9" t="inlineStr">
+        <is>
+          <t>quiz</t>
+        </is>
+      </c>
+      <c r="X95" s="9" t="inlineStr">
+        <is>
+          <t>퀴즈, 시험</t>
+        </is>
+      </c>
+      <c r="Y95" s="9" t="inlineStr">
+        <is>
+          <t>더블린 극장주 Daly가 무의미한 단어를 낙서하면 하루 만에 유행어로 만든 일화에서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-10
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y95"/>
+  <dimension ref="A1:Y96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11649,6 +11649,123 @@
         </is>
       </c>
     </row>
+    <row r="96" ht="60" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>단순과거 vs 과거진행</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>Past Simple vs Past Continuous</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F96" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H96" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I96" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Orpheus and Eurydice</t>
+        </is>
+      </c>
+      <c r="J96" s="9" t="inlineStr">
+        <is>
+          <t>Today we're looking at a classic Greek myth about Orpheus and Eurydice. This story teaches us about love and loss, and it's a great way to learn different uses of the word 'long'. The BBC has created a five-minute lesson that combines storytelling with vocabulary practice, so you can improve your English while enjoying a timeless tale.</t>
+        </is>
+      </c>
+      <c r="K96" s="9" t="inlineStr">
+        <is>
+          <t>combine — 결합하다; timeless — 시대를 초월한, 영원한</t>
+        </is>
+      </c>
+      <c r="L96" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M96" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N96" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O96" s="9" t="inlineStr">
+        <is>
+          <t>-s/-es 어미 발음 3가지</t>
+        </is>
+      </c>
+      <c r="P96" s="9" t="inlineStr">
+        <is>
+          <t>/ s/: 무성음 뒤 | /z/: 유성음 뒤 | /ɪz/: s·z·ch·sh로 끝날 때</t>
+        </is>
+      </c>
+      <c r="Q96" s="9" t="inlineStr">
+        <is>
+          <t>books /bʊks/ | dogs /dɒgz/ | watches /wɒtʃɪz/ | buses /bʌsɪz/</t>
+        </is>
+      </c>
+      <c r="R96" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S96" s="9" t="inlineStr"/>
+      <c r="T96" s="9" t="inlineStr"/>
+      <c r="U96" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V96" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W96" s="9" t="inlineStr">
+        <is>
+          <t>panic</t>
+        </is>
+      </c>
+      <c r="X96" s="9" t="inlineStr">
+        <is>
+          <t>공황, 극도의 공포</t>
+        </is>
+      </c>
+      <c r="Y96" s="9" t="inlineStr">
+        <is>
+          <t>목신 판(Pan)이 갑자기 나타나 공포를 일으킨다는 신화에서</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-11
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y96"/>
+  <dimension ref="A1:Y97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11766,6 +11766,123 @@
         </is>
       </c>
     </row>
+    <row r="97" ht="60" customHeight="1">
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B97" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C97" s="9" t="inlineStr">
+        <is>
+          <t>명사절과 간접의문문</t>
+        </is>
+      </c>
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>Noun Clauses and Embedded Questions</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G97" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H97" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I97" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pygmalion</t>
+        </is>
+      </c>
+      <c r="J97" s="9" t="inlineStr">
+        <is>
+          <t>Have you ever heard of Pygmalion? It's a classic story about an artist who falls in love with his own sculpture. Today we're going to explore this fascinating tale while learning eight different uses of the word 'round'. Stick around for five minutes and you'll pick up some really useful vocabulary!</t>
+        </is>
+      </c>
+      <c r="K97" s="9" t="inlineStr">
+        <is>
+          <t>sculpture — 조각상; stick around — 계속 머물다, 함께하다</t>
+        </is>
+      </c>
+      <c r="L97" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M97" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N97" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O97" s="9" t="inlineStr">
+        <is>
+          <t>연음 (Linking)</t>
+        </is>
+      </c>
+      <c r="P97" s="9" t="inlineStr">
+        <is>
+          <t>자음으로 끝나는 단어 + 모음으로 시작하는 단어는 이어서 발음</t>
+        </is>
+      </c>
+      <c r="Q97" s="9" t="inlineStr">
+        <is>
+          <t>pick it up → pi-ki-tup | turn it on → tur-ni-ton | look at it → loo-ka-tit</t>
+        </is>
+      </c>
+      <c r="R97" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S97" s="9" t="inlineStr"/>
+      <c r="T97" s="9" t="inlineStr"/>
+      <c r="U97" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V97" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W97" s="9" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="X97" s="9" t="inlineStr">
+        <is>
+          <t>전략</t>
+        </is>
+      </c>
+      <c r="Y97" s="9" t="inlineStr">
+        <is>
+          <t>stratos(군대) + agein(이끌다) → 장군의 기술</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily test page + learning log: 2026-09-12
</commit_message>
<xml_diff>
--- a/Improve_Eng/learning_log.xlsx
+++ b/Improve_Eng/learning_log.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y97"/>
+  <dimension ref="A1:Y98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11883,6 +11883,123 @@
         </is>
       </c>
     </row>
+    <row r="98" ht="60" customHeight="1">
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>현재완료 vs 단순과거</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>Present Perfect vs Simple Past</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>오늘 문법 규칙을 퀴즈 문제 해설에서 확인하세요.</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="inlineStr">
+        <is>
+          <t>I have worked here for five years.</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>① '어제' 같은 과거 시점과 현재완료 혼용 ② have+동사원형 실수</t>
+        </is>
+      </c>
+      <c r="H98" s="9" t="inlineStr">
+        <is>
+          <t>BBC Learning English Stories</t>
+        </is>
+      </c>
+      <c r="I98" s="9" t="inlineStr">
+        <is>
+          <t>Classic Stories: Pygmalion</t>
+        </is>
+      </c>
+      <c r="J98" s="9" t="inlineStr">
+        <is>
+          <t>Today we're exploring a classic story called Pygmalion, and we'll learn eight different uses of the word 'round.' The story teaches us about an artist who creates a perfect statue, and it's really engaging. So stick around for five minutes, and by the end, you'll understand how 'round' works in everyday English.</t>
+        </is>
+      </c>
+      <c r="K98" s="9" t="inlineStr">
+        <is>
+          <t>stick around — ~에 머물러 있다, 계속 함께하다; engaging — 흥미로운, 재미있는</t>
+        </is>
+      </c>
+      <c r="L98" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back</t>
+        </is>
+      </c>
+      <c r="M98" s="9" t="inlineStr">
+        <is>
+          <t>나중에 다시 돌아오다</t>
+        </is>
+      </c>
+      <c r="N98" s="9" t="inlineStr">
+        <is>
+          <t>Let's circle back on the budget after the Q2 data arrives.</t>
+        </is>
+      </c>
+      <c r="O98" s="9" t="inlineStr">
+        <is>
+          <t>약화 (Reduction)</t>
+        </is>
+      </c>
+      <c r="P98" s="9" t="inlineStr">
+        <is>
+          <t>기능어(of·to·for·and·at)는 빠르게 약화 — /ə/ 로 줄어듦</t>
+        </is>
+      </c>
+      <c r="Q98" s="9" t="inlineStr">
+        <is>
+          <t>cup of tea → cupə tea | a lot of → ə lɒtə | want to → wanna</t>
+        </is>
+      </c>
+      <c r="R98" s="9" t="inlineStr">
+        <is>
+          <t>allocate — 할당하다, 배정하다  |  allocate resources / allocate time / allocate budget</t>
+        </is>
+      </c>
+      <c r="S98" s="9" t="inlineStr"/>
+      <c r="T98" s="9" t="inlineStr"/>
+      <c r="U98" s="9" t="inlineStr">
+        <is>
+          <t>Topic Sentence 스캔</t>
+        </is>
+      </c>
+      <c r="V98" s="9" t="inlineStr">
+        <is>
+          <t>The global economy has shown signs of recovery. Consumer spending increased by 3% last quarter. However, inflation remains a concern for policymakers.</t>
+        </is>
+      </c>
+      <c r="W98" s="9" t="inlineStr">
+        <is>
+          <t>focus</t>
+        </is>
+      </c>
+      <c r="X98" s="9" t="inlineStr">
+        <is>
+          <t>초점, 집중</t>
+        </is>
+      </c>
+      <c r="Y98" s="9" t="inlineStr">
+        <is>
+          <t>로마 가정의 화덕이 집의 중심이었던 데서 유래</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>